<commit_message>
made some small changes
</commit_message>
<xml_diff>
--- a/USE_THIS_DESIGN_CODE/Input Excel Sheets/Mission Profiles/SD_Mission_Profile_Preliminary_Design.xlsx
+++ b/USE_THIS_DESIGN_CODE/Input Excel Sheets/Mission Profiles/SD_Mission_Profile_Preliminary_Design.xlsx
@@ -8,16 +8,17 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/zackwoj/Documents/MATLAB/26-27/Fall/Aircraft Design/Team06_SeniorProj/USE_THIS_DESIGN_CODE/Input Excel Sheets/Mission Profiles/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{061BE3F8-BC0C-D840-B8F5-53F9D4667016}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB20BF2F-D259-CB43-BB09-6BCE6F8C26F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16220" activeTab="1" xr2:uid="{AC12A90C-16A5-0547-A6DB-57534C200D25}"/>
   </bookViews>
   <sheets>
     <sheet name="Templates" sheetId="2" r:id="rId1"/>
     <sheet name="JB_{V1}" sheetId="13" r:id="rId2"/>
-    <sheet name="JB_{V1}_150mph_1hr" sheetId="15" r:id="rId3"/>
-    <sheet name="C172" sheetId="5" r:id="rId4"/>
-    <sheet name="Electric C172" sheetId="6" r:id="rId5"/>
+    <sheet name="JB_{V1}_ThresholdMaxM" sheetId="16" r:id="rId3"/>
+    <sheet name="JB_{V1}_150mph_1hr" sheetId="15" r:id="rId4"/>
+    <sheet name="C172" sheetId="5" r:id="rId5"/>
+    <sheet name="Electric C172" sheetId="6" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="199" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="244" uniqueCount="39">
   <si>
     <t>Takeoff</t>
   </si>
@@ -441,7 +442,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="44" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -476,12 +477,434 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Currency" xfId="1" builtinId="4"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="68">
+  <dxfs count="87">
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Arial Unicode MS"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="medium">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Arial Unicode MS"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Arial Unicode MS"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Arial Unicode MS"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Arial Unicode MS"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Arial Unicode MS"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Arial Unicode MS"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Arial Unicode MS"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Arial Unicode MS"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Arial Unicode MS"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="medium">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="medium">
+          <color rgb="FF000000"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <name val="Arial Unicode MS"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Arial Unicode MS"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+    </dxf>
     <dxf>
       <font>
         <b/>
@@ -1819,57 +2242,76 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{9C530343-8F22-3F4B-A21B-7146C98EA73F}" name="Table32352" displayName="Table32352" ref="A1:J200" totalsRowShown="0" headerRowDxfId="67" dataDxfId="66" tableBorderDxfId="65">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{9C530343-8F22-3F4B-A21B-7146C98EA73F}" name="Table32352" displayName="Table32352" ref="A1:J200" totalsRowShown="0" headerRowDxfId="86" dataDxfId="85" tableBorderDxfId="84">
   <autoFilter ref="A1:J200" xr:uid="{9C530343-8F22-3F4B-A21B-7146C98EA73F}"/>
   <tableColumns count="10">
-    <tableColumn id="1" xr3:uid="{1DCE1C02-B81F-5A42-9F8D-CD4F2F5FA0E1}" name="Segment #" dataDxfId="64"/>
-    <tableColumn id="2" xr3:uid="{5BC906B8-6517-EF46-B234-4259BF6806AC}" name="Segment Type" dataDxfId="63"/>
-    <tableColumn id="3" xr3:uid="{2316AD57-00CB-1E49-8500-2FF3F364AA6A}" name="Input 1" dataDxfId="62"/>
-    <tableColumn id="4" xr3:uid="{7B8395BD-D411-0042-9A31-EA5C362163AA}" name="Input 2" dataDxfId="61"/>
-    <tableColumn id="5" xr3:uid="{33A57DAD-EC47-2849-978C-EB31BD2A52E2}" name="Input 3" dataDxfId="60"/>
-    <tableColumn id="6" xr3:uid="{0A0C4CA9-5EB2-A241-9E5D-369C3DF8DD43}" name="Input 4" dataDxfId="59"/>
-    <tableColumn id="7" xr3:uid="{F74535B0-48DE-764E-BF99-0B508A958BAF}" name="Input 5" dataDxfId="58"/>
-    <tableColumn id="8" xr3:uid="{E9628660-11E2-3E40-A190-AD9EAF0C192F}" name="Input 6" dataDxfId="57"/>
-    <tableColumn id="9" xr3:uid="{EEA218E2-389D-1747-84AD-258E65EE195D}" name="Input 7" dataDxfId="56"/>
-    <tableColumn id="10" xr3:uid="{C68BB87A-98DA-5746-906B-34304D19B708}" name="Input 8" dataDxfId="55"/>
+    <tableColumn id="1" xr3:uid="{1DCE1C02-B81F-5A42-9F8D-CD4F2F5FA0E1}" name="Segment #" dataDxfId="83"/>
+    <tableColumn id="2" xr3:uid="{5BC906B8-6517-EF46-B234-4259BF6806AC}" name="Segment Type" dataDxfId="82"/>
+    <tableColumn id="3" xr3:uid="{2316AD57-00CB-1E49-8500-2FF3F364AA6A}" name="Input 1" dataDxfId="81"/>
+    <tableColumn id="4" xr3:uid="{7B8395BD-D411-0042-9A31-EA5C362163AA}" name="Input 2" dataDxfId="80"/>
+    <tableColumn id="5" xr3:uid="{33A57DAD-EC47-2849-978C-EB31BD2A52E2}" name="Input 3" dataDxfId="79"/>
+    <tableColumn id="6" xr3:uid="{0A0C4CA9-5EB2-A241-9E5D-369C3DF8DD43}" name="Input 4" dataDxfId="78"/>
+    <tableColumn id="7" xr3:uid="{F74535B0-48DE-764E-BF99-0B508A958BAF}" name="Input 5" dataDxfId="77"/>
+    <tableColumn id="8" xr3:uid="{E9628660-11E2-3E40-A190-AD9EAF0C192F}" name="Input 6" dataDxfId="76"/>
+    <tableColumn id="9" xr3:uid="{EEA218E2-389D-1747-84AD-258E65EE195D}" name="Input 7" dataDxfId="75"/>
+    <tableColumn id="10" xr3:uid="{C68BB87A-98DA-5746-906B-34304D19B708}" name="Input 8" dataDxfId="74"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium15" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{16BC0256-ADD7-EB41-B23C-2F629B8A0667}" name="Table323" displayName="Table323" ref="A1:J200" totalsRowShown="0" headerRowDxfId="54" dataDxfId="53" tableBorderDxfId="52">
-  <autoFilter ref="A1:J200" xr:uid="{E9D8E600-FE9F-5C45-8634-0D6DD0E667E3}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{09152E2F-423E-2F46-9775-46EEE677490E}" name="Table323524" displayName="Table323524" ref="A1:J200" totalsRowShown="0" headerRowDxfId="12" dataDxfId="11" tableBorderDxfId="10">
+  <autoFilter ref="A1:J200" xr:uid="{9C530343-8F22-3F4B-A21B-7146C98EA73F}"/>
   <tableColumns count="10">
-    <tableColumn id="1" xr3:uid="{D23BA427-6FDC-6C46-AADC-76777DF0599D}" name="Segment #" dataDxfId="51"/>
-    <tableColumn id="2" xr3:uid="{AF07C20E-012B-4A4D-9685-4B5C108A0C48}" name="Segment Type" dataDxfId="50"/>
-    <tableColumn id="3" xr3:uid="{4435643B-BB1E-B147-82C8-67CCC931376A}" name="Input 1" dataDxfId="49"/>
-    <tableColumn id="4" xr3:uid="{0B4DDA9A-2037-CD43-BDB5-1B7EC266CFA6}" name="Input 2" dataDxfId="48"/>
-    <tableColumn id="5" xr3:uid="{86FFB808-2BA0-844B-8C45-E32051CFF226}" name="Input 3" dataDxfId="47"/>
-    <tableColumn id="6" xr3:uid="{F128F1FB-77A9-344F-BFE0-756AD971F3AA}" name="Input 4" dataDxfId="46"/>
-    <tableColumn id="7" xr3:uid="{FC13F1AE-660A-024C-9FD6-B2953ADD8A85}" name="Input 5" dataDxfId="45"/>
-    <tableColumn id="8" xr3:uid="{3E1346B8-FB5C-6842-91DE-8C95912BEF7C}" name="Input 6" dataDxfId="44"/>
-    <tableColumn id="9" xr3:uid="{C19B4E6F-21EC-B346-A54F-D52512B94A8A}" name="Input 7" dataDxfId="43"/>
-    <tableColumn id="10" xr3:uid="{6524E215-8B7D-1E43-A2C0-2C1B780A18A9}" name="Input 8" dataDxfId="42"/>
+    <tableColumn id="1" xr3:uid="{980F29A0-8623-A445-9E6C-7FC765BBF570}" name="Segment #" dataDxfId="9"/>
+    <tableColumn id="2" xr3:uid="{8C5B23FC-4EB0-C941-8D07-22087992AA8F}" name="Segment Type" dataDxfId="8"/>
+    <tableColumn id="3" xr3:uid="{5798A81B-FB96-BA4C-9E78-BBAEC3A545AF}" name="Input 1" dataDxfId="7"/>
+    <tableColumn id="4" xr3:uid="{9EFC7076-6124-A94A-B30B-0AE379C26A23}" name="Input 2" dataDxfId="6"/>
+    <tableColumn id="5" xr3:uid="{615CB506-39EE-2345-95B7-5026BD89AA8D}" name="Input 3" dataDxfId="5"/>
+    <tableColumn id="6" xr3:uid="{F9EADA15-ECF7-A948-9CA1-32EB31E1A787}" name="Input 4" dataDxfId="4"/>
+    <tableColumn id="7" xr3:uid="{601B4314-7656-604A-B4A0-DDDDA1A6E0DF}" name="Input 5" dataDxfId="3"/>
+    <tableColumn id="8" xr3:uid="{F74CB3CC-5A53-BB47-A795-2FD7F77CA88C}" name="Input 6" dataDxfId="2"/>
+    <tableColumn id="9" xr3:uid="{4DE5B69B-C9D7-E84B-ACE2-A013B4F9F8C8}" name="Input 7" dataDxfId="1"/>
+    <tableColumn id="10" xr3:uid="{9E1DAD46-FA54-9F47-A684-D3188111C975}" name="Input 8" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium15" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{76C479A7-D97E-3440-915F-4416140AAFD6}" name="Table3235" displayName="Table3235" ref="A1:J200" totalsRowShown="0" headerRowDxfId="41" dataDxfId="40" tableBorderDxfId="39">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{16BC0256-ADD7-EB41-B23C-2F629B8A0667}" name="Table323" displayName="Table323" ref="A1:J200" totalsRowShown="0" headerRowDxfId="73" dataDxfId="72" tableBorderDxfId="71">
   <autoFilter ref="A1:J200" xr:uid="{E9D8E600-FE9F-5C45-8634-0D6DD0E667E3}"/>
   <tableColumns count="10">
-    <tableColumn id="1" xr3:uid="{15EB4EF6-08A8-964E-ABD5-0CF3EEC0C7B7}" name="Segment #" dataDxfId="38"/>
-    <tableColumn id="2" xr3:uid="{10C18371-46B8-6544-9972-D21BFA1DB0CD}" name="Segment Type" dataDxfId="37"/>
-    <tableColumn id="3" xr3:uid="{526667C5-306E-7D43-B338-699328AA6680}" name="Input 1" dataDxfId="36"/>
-    <tableColumn id="4" xr3:uid="{285F1D9C-6790-F049-8810-78F8A349CEA8}" name="Input 2" dataDxfId="35"/>
-    <tableColumn id="5" xr3:uid="{414CB0C1-F49D-4248-9E2F-428FEB38D5DA}" name="Input 3" dataDxfId="34"/>
-    <tableColumn id="6" xr3:uid="{7993028E-EBAF-D840-BAB7-8BA72340BA98}" name="Input 4" dataDxfId="33"/>
-    <tableColumn id="7" xr3:uid="{6617A981-14C9-8C42-A72A-0EB397E2F530}" name="Input 5" dataDxfId="32"/>
-    <tableColumn id="8" xr3:uid="{7AE9ECDF-5690-DE42-BC09-5934349F52E2}" name="Input 6" dataDxfId="31"/>
-    <tableColumn id="9" xr3:uid="{D1E2BD85-064E-C746-9E9E-6DA887B3E2CA}" name="Input 7" dataDxfId="30"/>
-    <tableColumn id="10" xr3:uid="{F7213638-D701-E04E-A444-9564EC9CA3EE}" name="Input 8" dataDxfId="29"/>
+    <tableColumn id="1" xr3:uid="{D23BA427-6FDC-6C46-AADC-76777DF0599D}" name="Segment #" dataDxfId="70"/>
+    <tableColumn id="2" xr3:uid="{AF07C20E-012B-4A4D-9685-4B5C108A0C48}" name="Segment Type" dataDxfId="69"/>
+    <tableColumn id="3" xr3:uid="{4435643B-BB1E-B147-82C8-67CCC931376A}" name="Input 1" dataDxfId="68"/>
+    <tableColumn id="4" xr3:uid="{0B4DDA9A-2037-CD43-BDB5-1B7EC266CFA6}" name="Input 2" dataDxfId="67"/>
+    <tableColumn id="5" xr3:uid="{86FFB808-2BA0-844B-8C45-E32051CFF226}" name="Input 3" dataDxfId="66"/>
+    <tableColumn id="6" xr3:uid="{F128F1FB-77A9-344F-BFE0-756AD971F3AA}" name="Input 4" dataDxfId="65"/>
+    <tableColumn id="7" xr3:uid="{FC13F1AE-660A-024C-9FD6-B2953ADD8A85}" name="Input 5" dataDxfId="64"/>
+    <tableColumn id="8" xr3:uid="{3E1346B8-FB5C-6842-91DE-8C95912BEF7C}" name="Input 6" dataDxfId="63"/>
+    <tableColumn id="9" xr3:uid="{C19B4E6F-21EC-B346-A54F-D52512B94A8A}" name="Input 7" dataDxfId="62"/>
+    <tableColumn id="10" xr3:uid="{6524E215-8B7D-1E43-A2C0-2C1B780A18A9}" name="Input 8" dataDxfId="61"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium15" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{76C479A7-D97E-3440-915F-4416140AAFD6}" name="Table3235" displayName="Table3235" ref="A1:J200" totalsRowShown="0" headerRowDxfId="60" dataDxfId="59" tableBorderDxfId="58">
+  <autoFilter ref="A1:J200" xr:uid="{E9D8E600-FE9F-5C45-8634-0D6DD0E667E3}"/>
+  <tableColumns count="10">
+    <tableColumn id="1" xr3:uid="{15EB4EF6-08A8-964E-ABD5-0CF3EEC0C7B7}" name="Segment #" dataDxfId="57"/>
+    <tableColumn id="2" xr3:uid="{10C18371-46B8-6544-9972-D21BFA1DB0CD}" name="Segment Type" dataDxfId="56"/>
+    <tableColumn id="3" xr3:uid="{526667C5-306E-7D43-B338-699328AA6680}" name="Input 1" dataDxfId="55"/>
+    <tableColumn id="4" xr3:uid="{285F1D9C-6790-F049-8810-78F8A349CEA8}" name="Input 2" dataDxfId="54"/>
+    <tableColumn id="5" xr3:uid="{414CB0C1-F49D-4248-9E2F-428FEB38D5DA}" name="Input 3" dataDxfId="53"/>
+    <tableColumn id="6" xr3:uid="{7993028E-EBAF-D840-BAB7-8BA72340BA98}" name="Input 4" dataDxfId="52"/>
+    <tableColumn id="7" xr3:uid="{6617A981-14C9-8C42-A72A-0EB397E2F530}" name="Input 5" dataDxfId="51"/>
+    <tableColumn id="8" xr3:uid="{7AE9ECDF-5690-DE42-BC09-5934349F52E2}" name="Input 6" dataDxfId="50"/>
+    <tableColumn id="9" xr3:uid="{D1E2BD85-064E-C746-9E9E-6DA887B3E2CA}" name="Input 7" dataDxfId="49"/>
+    <tableColumn id="10" xr3:uid="{F7213638-D701-E04E-A444-9564EC9CA3EE}" name="Input 8" dataDxfId="48"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium15" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2523,12 +2965,12 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A25:E26">
-    <cfRule type="expression" dxfId="28" priority="1">
+    <cfRule type="expression" dxfId="47" priority="1">
       <formula>MOD(ROW(),2)=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B1:F12 F13:F20 B15:E20 A21:F21 B22:F23">
-    <cfRule type="expression" dxfId="27" priority="2">
+    <cfRule type="expression" dxfId="46" priority="2">
       <formula>MOD(ROW(),2)=0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -2790,7 +3232,7 @@
         <v>13000</v>
       </c>
       <c r="D11" s="3">
-        <v>85</v>
+        <v>100</v>
       </c>
       <c r="E11" s="3">
         <v>0.1</v>
@@ -5108,32 +5550,32 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A1:A2 F2:J3 H4:J7 F12:J19 B2:E7 F4:F7 B8:J11">
-    <cfRule type="expression" dxfId="26" priority="7">
+    <cfRule type="expression" dxfId="45" priority="7">
       <formula>MOD(ROW(),2)=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B1 D1:J1">
-    <cfRule type="expression" dxfId="25" priority="8">
+    <cfRule type="expression" dxfId="44" priority="8">
       <formula>MOD(ROW(),2)=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B12:D13">
-    <cfRule type="expression" dxfId="24" priority="4">
+    <cfRule type="expression" dxfId="43" priority="4">
       <formula>MOD(ROW(),2)=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E12:E15">
-    <cfRule type="expression" dxfId="23" priority="3">
+    <cfRule type="expression" dxfId="42" priority="3">
       <formula>MOD(ROW(),2)=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E20:J21 A22:J200">
-    <cfRule type="expression" dxfId="22" priority="9">
+    <cfRule type="expression" dxfId="41" priority="9">
       <formula>MOD(ROW(),2)=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G4:G7">
-    <cfRule type="expression" dxfId="21" priority="6">
+    <cfRule type="expression" dxfId="40" priority="6">
       <formula>MOD(ROW(),2)=0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -5145,51 +5587,2662 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0628BF2E-9D96-DD48-8346-DBCC1EF66166}">
+  <dimension ref="A1:J200"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:10" ht="19" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A2" s="16">
+        <v>1</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="F2" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="G2" s="5"/>
+      <c r="H2" s="5"/>
+      <c r="I2" s="5"/>
+      <c r="J2" s="7"/>
+    </row>
+    <row r="3" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A3" s="8"/>
+      <c r="B3" s="3"/>
+      <c r="C3" s="3">
+        <v>8000</v>
+      </c>
+      <c r="D3" s="3">
+        <v>2</v>
+      </c>
+      <c r="E3" s="3">
+        <v>0.05</v>
+      </c>
+      <c r="F3" s="3">
+        <v>1.5E-3</v>
+      </c>
+      <c r="G3" s="3"/>
+      <c r="H3" s="3"/>
+      <c r="I3" s="3"/>
+      <c r="J3" s="9"/>
+    </row>
+    <row r="4" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A4" s="8">
+        <f>A2+1</f>
+        <v>2</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="H4" s="3"/>
+      <c r="I4" s="3"/>
+      <c r="J4" s="9"/>
+    </row>
+    <row r="5" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A5" s="8"/>
+      <c r="B5" s="3"/>
+      <c r="C5" s="3">
+        <v>8000</v>
+      </c>
+      <c r="D5" s="3">
+        <v>13000</v>
+      </c>
+      <c r="E5" s="3">
+        <v>4.7300000000000002E-2</v>
+      </c>
+      <c r="F5" s="3">
+        <v>0.1</v>
+      </c>
+      <c r="G5" s="3">
+        <v>0</v>
+      </c>
+      <c r="H5" s="3"/>
+      <c r="I5" s="3"/>
+      <c r="J5" s="9"/>
+    </row>
+    <row r="6" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A6" s="8">
+        <f>A4+1</f>
+        <v>3</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="G6" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="H6" s="3"/>
+      <c r="I6" s="3"/>
+      <c r="J6" s="9"/>
+    </row>
+    <row r="7" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A7" s="8"/>
+      <c r="B7" s="3"/>
+      <c r="C7" s="3">
+        <v>13000</v>
+      </c>
+      <c r="D7" s="3">
+        <v>15000</v>
+      </c>
+      <c r="E7" s="3">
+        <v>0.1</v>
+      </c>
+      <c r="F7" s="3">
+        <v>0.17</v>
+      </c>
+      <c r="G7" s="3">
+        <v>0</v>
+      </c>
+      <c r="H7" s="3"/>
+      <c r="I7" s="3"/>
+      <c r="J7" s="9"/>
+    </row>
+    <row r="8" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A8" s="8">
+        <v>4</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="G8" s="3"/>
+      <c r="H8" s="3"/>
+      <c r="I8" s="3"/>
+      <c r="J8" s="9"/>
+    </row>
+    <row r="9" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A9" s="8"/>
+      <c r="B9" s="3"/>
+      <c r="C9" s="3">
+        <v>15000</v>
+      </c>
+      <c r="D9" s="3">
+        <v>125</v>
+      </c>
+      <c r="E9" s="3">
+        <v>0.17</v>
+      </c>
+      <c r="F9" s="3">
+        <v>0</v>
+      </c>
+      <c r="G9" s="3"/>
+      <c r="H9" s="3"/>
+      <c r="I9" s="3"/>
+      <c r="J9" s="9"/>
+    </row>
+    <row r="10" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A10" s="8">
+        <v>5</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F10" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="G10" s="3"/>
+      <c r="H10" s="3"/>
+      <c r="I10" s="3"/>
+      <c r="J10" s="9"/>
+    </row>
+    <row r="11" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A11" s="8"/>
+      <c r="B11" s="3"/>
+      <c r="C11" s="3">
+        <v>13000</v>
+      </c>
+      <c r="D11" s="3">
+        <v>20</v>
+      </c>
+      <c r="E11" s="3">
+        <v>0.1</v>
+      </c>
+      <c r="F11" s="3">
+        <v>0</v>
+      </c>
+      <c r="G11" s="3"/>
+      <c r="H11" s="3"/>
+      <c r="I11" s="3"/>
+      <c r="J11" s="9"/>
+    </row>
+    <row r="12" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A12" s="8">
+        <v>6</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="F12" s="3"/>
+      <c r="G12" s="3"/>
+      <c r="H12" s="3"/>
+      <c r="I12" s="3"/>
+      <c r="J12" s="9"/>
+    </row>
+    <row r="13" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A13" s="8"/>
+      <c r="B13" s="3"/>
+      <c r="C13" s="14">
+        <v>13000</v>
+      </c>
+      <c r="D13" s="13">
+        <f>10/60</f>
+        <v>0.16666666666666666</v>
+      </c>
+      <c r="E13" s="3">
+        <v>0</v>
+      </c>
+      <c r="F13" s="3"/>
+      <c r="G13" s="3"/>
+      <c r="H13" s="3"/>
+      <c r="I13" s="3"/>
+      <c r="J13" s="9"/>
+    </row>
+    <row r="14" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A14" s="8">
+        <f>A12+1</f>
+        <v>7</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="D14" s="3"/>
+      <c r="E14" s="3"/>
+      <c r="F14" s="4"/>
+      <c r="G14" s="3"/>
+      <c r="H14" s="3"/>
+      <c r="I14" s="3"/>
+      <c r="J14" s="9"/>
+    </row>
+    <row r="15" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A15" s="8"/>
+      <c r="B15" s="3"/>
+      <c r="C15" s="3">
+        <v>0.01</v>
+      </c>
+      <c r="D15" s="3"/>
+      <c r="E15" s="3"/>
+      <c r="F15" s="3"/>
+      <c r="G15" s="3"/>
+      <c r="H15" s="3"/>
+      <c r="I15" s="3"/>
+      <c r="J15" s="9"/>
+    </row>
+    <row r="16" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A16" s="8">
+        <f>A14+1</f>
+        <v>8</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="D16" s="3"/>
+      <c r="E16" s="3"/>
+      <c r="F16" s="3"/>
+      <c r="G16" s="3"/>
+      <c r="H16" s="3"/>
+      <c r="I16" s="3"/>
+      <c r="J16" s="9"/>
+    </row>
+    <row r="17" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A17" s="8"/>
+      <c r="B17" s="3"/>
+      <c r="C17" s="3">
+        <v>1E-4</v>
+      </c>
+      <c r="D17" s="3"/>
+      <c r="E17" s="3"/>
+      <c r="F17" s="3"/>
+      <c r="G17" s="3"/>
+      <c r="H17" s="3"/>
+      <c r="I17" s="3"/>
+      <c r="J17" s="9"/>
+    </row>
+    <row r="18" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A18" s="8"/>
+      <c r="B18" s="4"/>
+      <c r="C18" s="4"/>
+      <c r="D18" s="3"/>
+      <c r="E18" s="3"/>
+      <c r="F18" s="3"/>
+      <c r="G18" s="3"/>
+      <c r="H18" s="3"/>
+      <c r="I18" s="3"/>
+      <c r="J18" s="9"/>
+    </row>
+    <row r="19" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A19" s="8"/>
+      <c r="B19" s="3"/>
+      <c r="C19" s="3"/>
+      <c r="D19" s="3"/>
+      <c r="E19" s="3"/>
+      <c r="F19" s="3"/>
+      <c r="G19" s="3"/>
+      <c r="H19" s="3"/>
+      <c r="I19" s="3"/>
+      <c r="J19" s="9"/>
+    </row>
+    <row r="20" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A20" s="8"/>
+      <c r="B20" s="3"/>
+      <c r="C20" s="3"/>
+      <c r="D20" s="3"/>
+      <c r="E20" s="3"/>
+      <c r="F20" s="3"/>
+      <c r="G20" s="3"/>
+      <c r="H20" s="3"/>
+      <c r="I20" s="3"/>
+      <c r="J20" s="9"/>
+    </row>
+    <row r="21" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A21" s="6"/>
+      <c r="B21" s="3"/>
+      <c r="C21" s="3"/>
+      <c r="D21" s="3"/>
+      <c r="E21" s="3"/>
+      <c r="F21" s="3"/>
+      <c r="G21" s="3"/>
+      <c r="H21" s="3"/>
+      <c r="I21" s="3"/>
+      <c r="J21" s="9"/>
+    </row>
+    <row r="22" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A22" s="6"/>
+      <c r="B22" s="3"/>
+      <c r="C22" s="3"/>
+      <c r="D22" s="3"/>
+      <c r="E22" s="3"/>
+      <c r="F22" s="3"/>
+      <c r="G22" s="3"/>
+      <c r="H22" s="3"/>
+      <c r="I22" s="3"/>
+      <c r="J22" s="9"/>
+    </row>
+    <row r="23" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A23" s="6"/>
+      <c r="B23" s="3"/>
+      <c r="C23" s="3"/>
+      <c r="D23" s="3"/>
+      <c r="E23" s="3"/>
+      <c r="F23" s="3"/>
+      <c r="G23" s="3"/>
+      <c r="H23" s="3"/>
+      <c r="I23" s="3"/>
+      <c r="J23" s="9"/>
+    </row>
+    <row r="24" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A24" s="6"/>
+      <c r="B24" s="3"/>
+      <c r="C24" s="3"/>
+      <c r="D24" s="3"/>
+      <c r="E24" s="3"/>
+      <c r="F24" s="3"/>
+      <c r="G24" s="3"/>
+      <c r="H24" s="3"/>
+      <c r="I24" s="3"/>
+      <c r="J24" s="9"/>
+    </row>
+    <row r="25" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A25" s="6"/>
+      <c r="B25" s="3"/>
+      <c r="C25" s="3"/>
+      <c r="D25" s="3"/>
+      <c r="E25" s="3"/>
+      <c r="F25" s="3"/>
+      <c r="G25" s="3"/>
+      <c r="H25" s="3"/>
+      <c r="I25" s="3"/>
+      <c r="J25" s="9"/>
+    </row>
+    <row r="26" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A26" s="6"/>
+      <c r="B26" s="3"/>
+      <c r="C26" s="3"/>
+      <c r="D26" s="3"/>
+      <c r="E26" s="3"/>
+      <c r="F26" s="3"/>
+      <c r="G26" s="3"/>
+      <c r="H26" s="3"/>
+      <c r="I26" s="3"/>
+      <c r="J26" s="9"/>
+    </row>
+    <row r="27" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A27" s="6"/>
+      <c r="B27" s="3"/>
+      <c r="C27" s="3"/>
+      <c r="D27" s="3"/>
+      <c r="E27" s="3"/>
+      <c r="F27" s="3"/>
+      <c r="G27" s="3"/>
+      <c r="H27" s="3"/>
+      <c r="I27" s="3"/>
+      <c r="J27" s="9"/>
+    </row>
+    <row r="28" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A28" s="6"/>
+      <c r="B28" s="3"/>
+      <c r="C28" s="3"/>
+      <c r="D28" s="3"/>
+      <c r="E28" s="3"/>
+      <c r="F28" s="3"/>
+      <c r="G28" s="3"/>
+      <c r="H28" s="3"/>
+      <c r="I28" s="3"/>
+      <c r="J28" s="9"/>
+    </row>
+    <row r="29" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A29" s="6"/>
+      <c r="B29" s="3"/>
+      <c r="C29" s="3"/>
+      <c r="D29" s="3"/>
+      <c r="E29" s="3"/>
+      <c r="F29" s="3"/>
+      <c r="G29" s="3"/>
+      <c r="H29" s="3"/>
+      <c r="I29" s="3"/>
+      <c r="J29" s="9"/>
+    </row>
+    <row r="30" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A30" s="6"/>
+      <c r="B30" s="3"/>
+      <c r="C30" s="3"/>
+      <c r="D30" s="3"/>
+      <c r="E30" s="3"/>
+      <c r="F30" s="3"/>
+      <c r="G30" s="3"/>
+      <c r="H30" s="3"/>
+      <c r="I30" s="3"/>
+      <c r="J30" s="9"/>
+    </row>
+    <row r="31" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A31" s="6"/>
+      <c r="B31" s="3"/>
+      <c r="C31" s="3"/>
+      <c r="D31" s="3"/>
+      <c r="E31" s="3"/>
+      <c r="F31" s="3"/>
+      <c r="G31" s="3"/>
+      <c r="H31" s="3"/>
+      <c r="I31" s="3"/>
+      <c r="J31" s="9"/>
+    </row>
+    <row r="32" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A32" s="6"/>
+      <c r="B32" s="3"/>
+      <c r="C32" s="3"/>
+      <c r="D32" s="3"/>
+      <c r="E32" s="3"/>
+      <c r="F32" s="3"/>
+      <c r="G32" s="3"/>
+      <c r="H32" s="3"/>
+      <c r="I32" s="3"/>
+      <c r="J32" s="9"/>
+    </row>
+    <row r="33" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A33" s="6"/>
+      <c r="B33" s="3"/>
+      <c r="C33" s="3"/>
+      <c r="D33" s="3"/>
+      <c r="E33" s="3"/>
+      <c r="F33" s="3"/>
+      <c r="G33" s="3"/>
+      <c r="H33" s="3"/>
+      <c r="I33" s="3"/>
+      <c r="J33" s="9"/>
+    </row>
+    <row r="34" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A34" s="6"/>
+      <c r="B34" s="3"/>
+      <c r="C34" s="3"/>
+      <c r="D34" s="3"/>
+      <c r="E34" s="3"/>
+      <c r="F34" s="3"/>
+      <c r="G34" s="3"/>
+      <c r="H34" s="3"/>
+      <c r="I34" s="3"/>
+      <c r="J34" s="9"/>
+    </row>
+    <row r="35" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A35" s="6"/>
+      <c r="B35" s="3"/>
+      <c r="C35" s="3"/>
+      <c r="D35" s="3"/>
+      <c r="E35" s="3"/>
+      <c r="F35" s="3"/>
+      <c r="G35" s="3"/>
+      <c r="H35" s="3"/>
+      <c r="I35" s="3"/>
+      <c r="J35" s="9"/>
+    </row>
+    <row r="36" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A36" s="6"/>
+      <c r="B36" s="3"/>
+      <c r="C36" s="3"/>
+      <c r="D36" s="3"/>
+      <c r="E36" s="3"/>
+      <c r="F36" s="3"/>
+      <c r="G36" s="3"/>
+      <c r="H36" s="3"/>
+      <c r="I36" s="3"/>
+      <c r="J36" s="9"/>
+    </row>
+    <row r="37" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A37" s="6"/>
+      <c r="B37" s="3"/>
+      <c r="C37" s="3"/>
+      <c r="D37" s="3"/>
+      <c r="E37" s="3"/>
+      <c r="F37" s="3"/>
+      <c r="G37" s="3"/>
+      <c r="H37" s="3"/>
+      <c r="I37" s="3"/>
+      <c r="J37" s="9"/>
+    </row>
+    <row r="38" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A38" s="6"/>
+      <c r="B38" s="3"/>
+      <c r="C38" s="3"/>
+      <c r="D38" s="3"/>
+      <c r="E38" s="3"/>
+      <c r="F38" s="3"/>
+      <c r="G38" s="3"/>
+      <c r="H38" s="3"/>
+      <c r="I38" s="3"/>
+      <c r="J38" s="9"/>
+    </row>
+    <row r="39" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A39" s="6"/>
+      <c r="B39" s="3"/>
+      <c r="C39" s="3"/>
+      <c r="D39" s="3"/>
+      <c r="E39" s="3"/>
+      <c r="F39" s="3"/>
+      <c r="G39" s="3"/>
+      <c r="H39" s="3"/>
+      <c r="I39" s="3"/>
+      <c r="J39" s="9"/>
+    </row>
+    <row r="40" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A40" s="6"/>
+      <c r="B40" s="3"/>
+      <c r="C40" s="3"/>
+      <c r="D40" s="3"/>
+      <c r="E40" s="3"/>
+      <c r="F40" s="3"/>
+      <c r="G40" s="3"/>
+      <c r="H40" s="3"/>
+      <c r="I40" s="3"/>
+      <c r="J40" s="9"/>
+    </row>
+    <row r="41" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A41" s="6"/>
+      <c r="B41" s="3"/>
+      <c r="C41" s="3"/>
+      <c r="D41" s="3"/>
+      <c r="E41" s="3"/>
+      <c r="F41" s="3"/>
+      <c r="G41" s="3"/>
+      <c r="H41" s="3"/>
+      <c r="I41" s="3"/>
+      <c r="J41" s="9"/>
+    </row>
+    <row r="42" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A42" s="6"/>
+      <c r="B42" s="3"/>
+      <c r="C42" s="3"/>
+      <c r="D42" s="3"/>
+      <c r="E42" s="3"/>
+      <c r="F42" s="3"/>
+      <c r="G42" s="3"/>
+      <c r="H42" s="3"/>
+      <c r="I42" s="3"/>
+      <c r="J42" s="9"/>
+    </row>
+    <row r="43" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A43" s="6"/>
+      <c r="B43" s="3"/>
+      <c r="C43" s="3"/>
+      <c r="D43" s="3"/>
+      <c r="E43" s="3"/>
+      <c r="F43" s="3"/>
+      <c r="G43" s="3"/>
+      <c r="H43" s="3"/>
+      <c r="I43" s="3"/>
+      <c r="J43" s="9"/>
+    </row>
+    <row r="44" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A44" s="6"/>
+      <c r="B44" s="3"/>
+      <c r="C44" s="3"/>
+      <c r="D44" s="3"/>
+      <c r="E44" s="3"/>
+      <c r="F44" s="3"/>
+      <c r="G44" s="3"/>
+      <c r="H44" s="3"/>
+      <c r="I44" s="3"/>
+      <c r="J44" s="9"/>
+    </row>
+    <row r="45" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A45" s="6"/>
+      <c r="B45" s="3"/>
+      <c r="C45" s="3"/>
+      <c r="D45" s="3"/>
+      <c r="E45" s="3"/>
+      <c r="F45" s="3"/>
+      <c r="G45" s="3"/>
+      <c r="H45" s="3"/>
+      <c r="I45" s="3"/>
+      <c r="J45" s="9"/>
+    </row>
+    <row r="46" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A46" s="6"/>
+      <c r="B46" s="3"/>
+      <c r="C46" s="3"/>
+      <c r="D46" s="3"/>
+      <c r="E46" s="3"/>
+      <c r="F46" s="3"/>
+      <c r="G46" s="3"/>
+      <c r="H46" s="3"/>
+      <c r="I46" s="3"/>
+      <c r="J46" s="9"/>
+    </row>
+    <row r="47" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A47" s="6"/>
+      <c r="B47" s="3"/>
+      <c r="C47" s="3"/>
+      <c r="D47" s="3"/>
+      <c r="E47" s="3"/>
+      <c r="F47" s="3"/>
+      <c r="G47" s="3"/>
+      <c r="H47" s="3"/>
+      <c r="I47" s="3"/>
+      <c r="J47" s="9"/>
+    </row>
+    <row r="48" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A48" s="6"/>
+      <c r="B48" s="3"/>
+      <c r="C48" s="3"/>
+      <c r="D48" s="3"/>
+      <c r="E48" s="3"/>
+      <c r="F48" s="3"/>
+      <c r="G48" s="3"/>
+      <c r="H48" s="3"/>
+      <c r="I48" s="3"/>
+      <c r="J48" s="9"/>
+    </row>
+    <row r="49" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A49" s="6"/>
+      <c r="B49" s="3"/>
+      <c r="C49" s="3"/>
+      <c r="D49" s="3"/>
+      <c r="E49" s="3"/>
+      <c r="F49" s="3"/>
+      <c r="G49" s="3"/>
+      <c r="H49" s="3"/>
+      <c r="I49" s="3"/>
+      <c r="J49" s="9"/>
+    </row>
+    <row r="50" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A50" s="6"/>
+      <c r="B50" s="3"/>
+      <c r="C50" s="3"/>
+      <c r="D50" s="3"/>
+      <c r="E50" s="3"/>
+      <c r="F50" s="3"/>
+      <c r="G50" s="3"/>
+      <c r="H50" s="3"/>
+      <c r="I50" s="3"/>
+      <c r="J50" s="9"/>
+    </row>
+    <row r="51" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A51" s="6"/>
+      <c r="B51" s="3"/>
+      <c r="C51" s="3"/>
+      <c r="D51" s="3"/>
+      <c r="E51" s="3"/>
+      <c r="F51" s="3"/>
+      <c r="G51" s="3"/>
+      <c r="H51" s="3"/>
+      <c r="I51" s="3"/>
+      <c r="J51" s="9"/>
+    </row>
+    <row r="52" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A52" s="6"/>
+      <c r="B52" s="3"/>
+      <c r="C52" s="3"/>
+      <c r="D52" s="3"/>
+      <c r="E52" s="3"/>
+      <c r="F52" s="3"/>
+      <c r="G52" s="3"/>
+      <c r="H52" s="3"/>
+      <c r="I52" s="3"/>
+      <c r="J52" s="9"/>
+    </row>
+    <row r="53" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A53" s="6"/>
+      <c r="B53" s="3"/>
+      <c r="C53" s="3"/>
+      <c r="D53" s="3"/>
+      <c r="E53" s="3"/>
+      <c r="F53" s="3"/>
+      <c r="G53" s="3"/>
+      <c r="H53" s="3"/>
+      <c r="I53" s="3"/>
+      <c r="J53" s="9"/>
+    </row>
+    <row r="54" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A54" s="6"/>
+      <c r="B54" s="3"/>
+      <c r="C54" s="3"/>
+      <c r="D54" s="3"/>
+      <c r="E54" s="3"/>
+      <c r="F54" s="3"/>
+      <c r="G54" s="3"/>
+      <c r="H54" s="3"/>
+      <c r="I54" s="3"/>
+      <c r="J54" s="9"/>
+    </row>
+    <row r="55" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A55" s="6"/>
+      <c r="B55" s="3"/>
+      <c r="C55" s="3"/>
+      <c r="D55" s="3"/>
+      <c r="E55" s="3"/>
+      <c r="F55" s="3"/>
+      <c r="G55" s="3"/>
+      <c r="H55" s="3"/>
+      <c r="I55" s="3"/>
+      <c r="J55" s="9"/>
+    </row>
+    <row r="56" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A56" s="6"/>
+      <c r="B56" s="3"/>
+      <c r="C56" s="3"/>
+      <c r="D56" s="3"/>
+      <c r="E56" s="3"/>
+      <c r="F56" s="3"/>
+      <c r="G56" s="3"/>
+      <c r="H56" s="3"/>
+      <c r="I56" s="3"/>
+      <c r="J56" s="9"/>
+    </row>
+    <row r="57" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A57" s="6"/>
+      <c r="B57" s="3"/>
+      <c r="C57" s="3"/>
+      <c r="D57" s="3"/>
+      <c r="E57" s="3"/>
+      <c r="F57" s="3"/>
+      <c r="G57" s="3"/>
+      <c r="H57" s="3"/>
+      <c r="I57" s="3"/>
+      <c r="J57" s="9"/>
+    </row>
+    <row r="58" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A58" s="6"/>
+      <c r="B58" s="3"/>
+      <c r="C58" s="3"/>
+      <c r="D58" s="3"/>
+      <c r="E58" s="3"/>
+      <c r="F58" s="3"/>
+      <c r="G58" s="3"/>
+      <c r="H58" s="3"/>
+      <c r="I58" s="3"/>
+      <c r="J58" s="9"/>
+    </row>
+    <row r="59" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A59" s="6"/>
+      <c r="B59" s="3"/>
+      <c r="C59" s="3"/>
+      <c r="D59" s="3"/>
+      <c r="E59" s="3"/>
+      <c r="F59" s="3"/>
+      <c r="G59" s="3"/>
+      <c r="H59" s="3"/>
+      <c r="I59" s="3"/>
+      <c r="J59" s="9"/>
+    </row>
+    <row r="60" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A60" s="6"/>
+      <c r="B60" s="3"/>
+      <c r="C60" s="3"/>
+      <c r="D60" s="3"/>
+      <c r="E60" s="3"/>
+      <c r="F60" s="3"/>
+      <c r="G60" s="3"/>
+      <c r="H60" s="3"/>
+      <c r="I60" s="3"/>
+      <c r="J60" s="9"/>
+    </row>
+    <row r="61" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A61" s="6"/>
+      <c r="B61" s="3"/>
+      <c r="C61" s="3"/>
+      <c r="D61" s="3"/>
+      <c r="E61" s="3"/>
+      <c r="F61" s="3"/>
+      <c r="G61" s="3"/>
+      <c r="H61" s="3"/>
+      <c r="I61" s="3"/>
+      <c r="J61" s="9"/>
+    </row>
+    <row r="62" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A62" s="6"/>
+      <c r="B62" s="3"/>
+      <c r="C62" s="3"/>
+      <c r="D62" s="3"/>
+      <c r="E62" s="3"/>
+      <c r="F62" s="3"/>
+      <c r="G62" s="3"/>
+      <c r="H62" s="3"/>
+      <c r="I62" s="3"/>
+      <c r="J62" s="9"/>
+    </row>
+    <row r="63" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A63" s="6"/>
+      <c r="B63" s="3"/>
+      <c r="C63" s="3"/>
+      <c r="D63" s="3"/>
+      <c r="E63" s="3"/>
+      <c r="F63" s="3"/>
+      <c r="G63" s="3"/>
+      <c r="H63" s="3"/>
+      <c r="I63" s="3"/>
+      <c r="J63" s="9"/>
+    </row>
+    <row r="64" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A64" s="6"/>
+      <c r="B64" s="3"/>
+      <c r="C64" s="3"/>
+      <c r="D64" s="3"/>
+      <c r="E64" s="3"/>
+      <c r="F64" s="3"/>
+      <c r="G64" s="3"/>
+      <c r="H64" s="3"/>
+      <c r="I64" s="3"/>
+      <c r="J64" s="9"/>
+    </row>
+    <row r="65" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A65" s="6"/>
+      <c r="B65" s="3"/>
+      <c r="C65" s="3"/>
+      <c r="D65" s="3"/>
+      <c r="E65" s="3"/>
+      <c r="F65" s="3"/>
+      <c r="G65" s="3"/>
+      <c r="H65" s="3"/>
+      <c r="I65" s="3"/>
+      <c r="J65" s="9"/>
+    </row>
+    <row r="66" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A66" s="6"/>
+      <c r="B66" s="3"/>
+      <c r="C66" s="3"/>
+      <c r="D66" s="3"/>
+      <c r="E66" s="3"/>
+      <c r="F66" s="3"/>
+      <c r="G66" s="3"/>
+      <c r="H66" s="3"/>
+      <c r="I66" s="3"/>
+      <c r="J66" s="9"/>
+    </row>
+    <row r="67" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A67" s="6"/>
+      <c r="B67" s="3"/>
+      <c r="C67" s="3"/>
+      <c r="D67" s="3"/>
+      <c r="E67" s="3"/>
+      <c r="F67" s="3"/>
+      <c r="G67" s="3"/>
+      <c r="H67" s="3"/>
+      <c r="I67" s="3"/>
+      <c r="J67" s="9"/>
+    </row>
+    <row r="68" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A68" s="6"/>
+      <c r="B68" s="3"/>
+      <c r="C68" s="3"/>
+      <c r="D68" s="3"/>
+      <c r="E68" s="3"/>
+      <c r="F68" s="3"/>
+      <c r="G68" s="3"/>
+      <c r="H68" s="3"/>
+      <c r="I68" s="3"/>
+      <c r="J68" s="9"/>
+    </row>
+    <row r="69" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A69" s="6"/>
+      <c r="B69" s="3"/>
+      <c r="C69" s="3"/>
+      <c r="D69" s="3"/>
+      <c r="E69" s="3"/>
+      <c r="F69" s="3"/>
+      <c r="G69" s="3"/>
+      <c r="H69" s="3"/>
+      <c r="I69" s="3"/>
+      <c r="J69" s="9"/>
+    </row>
+    <row r="70" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A70" s="6"/>
+      <c r="B70" s="3"/>
+      <c r="C70" s="3"/>
+      <c r="D70" s="3"/>
+      <c r="E70" s="3"/>
+      <c r="F70" s="3"/>
+      <c r="G70" s="3"/>
+      <c r="H70" s="3"/>
+      <c r="I70" s="3"/>
+      <c r="J70" s="9"/>
+    </row>
+    <row r="71" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A71" s="6"/>
+      <c r="B71" s="3"/>
+      <c r="C71" s="3"/>
+      <c r="D71" s="3"/>
+      <c r="E71" s="3"/>
+      <c r="F71" s="3"/>
+      <c r="G71" s="3"/>
+      <c r="H71" s="3"/>
+      <c r="I71" s="3"/>
+      <c r="J71" s="9"/>
+    </row>
+    <row r="72" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A72" s="6"/>
+      <c r="B72" s="3"/>
+      <c r="C72" s="3"/>
+      <c r="D72" s="3"/>
+      <c r="E72" s="3"/>
+      <c r="F72" s="3"/>
+      <c r="G72" s="3"/>
+      <c r="H72" s="3"/>
+      <c r="I72" s="3"/>
+      <c r="J72" s="9"/>
+    </row>
+    <row r="73" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A73" s="6"/>
+      <c r="B73" s="3"/>
+      <c r="C73" s="3"/>
+      <c r="D73" s="3"/>
+      <c r="E73" s="3"/>
+      <c r="F73" s="3"/>
+      <c r="G73" s="3"/>
+      <c r="H73" s="3"/>
+      <c r="I73" s="3"/>
+      <c r="J73" s="9"/>
+    </row>
+    <row r="74" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A74" s="6"/>
+      <c r="B74" s="3"/>
+      <c r="C74" s="3"/>
+      <c r="D74" s="3"/>
+      <c r="E74" s="3"/>
+      <c r="F74" s="3"/>
+      <c r="G74" s="3"/>
+      <c r="H74" s="3"/>
+      <c r="I74" s="3"/>
+      <c r="J74" s="9"/>
+    </row>
+    <row r="75" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A75" s="6"/>
+      <c r="B75" s="3"/>
+      <c r="C75" s="3"/>
+      <c r="D75" s="3"/>
+      <c r="E75" s="3"/>
+      <c r="F75" s="3"/>
+      <c r="G75" s="3"/>
+      <c r="H75" s="3"/>
+      <c r="I75" s="3"/>
+      <c r="J75" s="9"/>
+    </row>
+    <row r="76" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A76" s="6"/>
+      <c r="B76" s="3"/>
+      <c r="C76" s="3"/>
+      <c r="D76" s="3"/>
+      <c r="E76" s="3"/>
+      <c r="F76" s="3"/>
+      <c r="G76" s="3"/>
+      <c r="H76" s="3"/>
+      <c r="I76" s="3"/>
+      <c r="J76" s="9"/>
+    </row>
+    <row r="77" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A77" s="6"/>
+      <c r="B77" s="3"/>
+      <c r="C77" s="3"/>
+      <c r="D77" s="3"/>
+      <c r="E77" s="3"/>
+      <c r="F77" s="3"/>
+      <c r="G77" s="3"/>
+      <c r="H77" s="3"/>
+      <c r="I77" s="3"/>
+      <c r="J77" s="9"/>
+    </row>
+    <row r="78" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A78" s="6"/>
+      <c r="B78" s="3"/>
+      <c r="C78" s="3"/>
+      <c r="D78" s="3"/>
+      <c r="E78" s="3"/>
+      <c r="F78" s="3"/>
+      <c r="G78" s="3"/>
+      <c r="H78" s="3"/>
+      <c r="I78" s="3"/>
+      <c r="J78" s="9"/>
+    </row>
+    <row r="79" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A79" s="6"/>
+      <c r="B79" s="3"/>
+      <c r="C79" s="3"/>
+      <c r="D79" s="3"/>
+      <c r="E79" s="3"/>
+      <c r="F79" s="3"/>
+      <c r="G79" s="3"/>
+      <c r="H79" s="3"/>
+      <c r="I79" s="3"/>
+      <c r="J79" s="9"/>
+    </row>
+    <row r="80" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A80" s="6"/>
+      <c r="B80" s="3"/>
+      <c r="C80" s="3"/>
+      <c r="D80" s="3"/>
+      <c r="E80" s="3"/>
+      <c r="F80" s="3"/>
+      <c r="G80" s="3"/>
+      <c r="H80" s="3"/>
+      <c r="I80" s="3"/>
+      <c r="J80" s="9"/>
+    </row>
+    <row r="81" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A81" s="6"/>
+      <c r="B81" s="3"/>
+      <c r="C81" s="3"/>
+      <c r="D81" s="3"/>
+      <c r="E81" s="3"/>
+      <c r="F81" s="3"/>
+      <c r="G81" s="3"/>
+      <c r="H81" s="3"/>
+      <c r="I81" s="3"/>
+      <c r="J81" s="9"/>
+    </row>
+    <row r="82" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A82" s="6"/>
+      <c r="B82" s="3"/>
+      <c r="C82" s="3"/>
+      <c r="D82" s="3"/>
+      <c r="E82" s="3"/>
+      <c r="F82" s="3"/>
+      <c r="G82" s="3"/>
+      <c r="H82" s="3"/>
+      <c r="I82" s="3"/>
+      <c r="J82" s="9"/>
+    </row>
+    <row r="83" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A83" s="6"/>
+      <c r="B83" s="3"/>
+      <c r="C83" s="3"/>
+      <c r="D83" s="3"/>
+      <c r="E83" s="3"/>
+      <c r="F83" s="3"/>
+      <c r="G83" s="3"/>
+      <c r="H83" s="3"/>
+      <c r="I83" s="3"/>
+      <c r="J83" s="9"/>
+    </row>
+    <row r="84" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A84" s="6"/>
+      <c r="B84" s="3"/>
+      <c r="C84" s="3"/>
+      <c r="D84" s="3"/>
+      <c r="E84" s="3"/>
+      <c r="F84" s="3"/>
+      <c r="G84" s="3"/>
+      <c r="H84" s="3"/>
+      <c r="I84" s="3"/>
+      <c r="J84" s="9"/>
+    </row>
+    <row r="85" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A85" s="6"/>
+      <c r="B85" s="3"/>
+      <c r="C85" s="3"/>
+      <c r="D85" s="3"/>
+      <c r="E85" s="3"/>
+      <c r="F85" s="3"/>
+      <c r="G85" s="3"/>
+      <c r="H85" s="3"/>
+      <c r="I85" s="3"/>
+      <c r="J85" s="9"/>
+    </row>
+    <row r="86" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A86" s="6"/>
+      <c r="B86" s="3"/>
+      <c r="C86" s="3"/>
+      <c r="D86" s="3"/>
+      <c r="E86" s="3"/>
+      <c r="F86" s="3"/>
+      <c r="G86" s="3"/>
+      <c r="H86" s="3"/>
+      <c r="I86" s="3"/>
+      <c r="J86" s="9"/>
+    </row>
+    <row r="87" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A87" s="6"/>
+      <c r="B87" s="3"/>
+      <c r="C87" s="3"/>
+      <c r="D87" s="3"/>
+      <c r="E87" s="3"/>
+      <c r="F87" s="3"/>
+      <c r="G87" s="3"/>
+      <c r="H87" s="3"/>
+      <c r="I87" s="3"/>
+      <c r="J87" s="9"/>
+    </row>
+    <row r="88" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A88" s="6"/>
+      <c r="B88" s="3"/>
+      <c r="C88" s="3"/>
+      <c r="D88" s="3"/>
+      <c r="E88" s="3"/>
+      <c r="F88" s="3"/>
+      <c r="G88" s="3"/>
+      <c r="H88" s="3"/>
+      <c r="I88" s="3"/>
+      <c r="J88" s="9"/>
+    </row>
+    <row r="89" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A89" s="6"/>
+      <c r="B89" s="3"/>
+      <c r="C89" s="3"/>
+      <c r="D89" s="3"/>
+      <c r="E89" s="3"/>
+      <c r="F89" s="3"/>
+      <c r="G89" s="3"/>
+      <c r="H89" s="3"/>
+      <c r="I89" s="3"/>
+      <c r="J89" s="9"/>
+    </row>
+    <row r="90" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A90" s="6"/>
+      <c r="B90" s="3"/>
+      <c r="C90" s="3"/>
+      <c r="D90" s="3"/>
+      <c r="E90" s="3"/>
+      <c r="F90" s="3"/>
+      <c r="G90" s="3"/>
+      <c r="H90" s="3"/>
+      <c r="I90" s="3"/>
+      <c r="J90" s="9"/>
+    </row>
+    <row r="91" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A91" s="6"/>
+      <c r="B91" s="3"/>
+      <c r="C91" s="3"/>
+      <c r="D91" s="3"/>
+      <c r="E91" s="3"/>
+      <c r="F91" s="3"/>
+      <c r="G91" s="3"/>
+      <c r="H91" s="3"/>
+      <c r="I91" s="3"/>
+      <c r="J91" s="9"/>
+    </row>
+    <row r="92" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A92" s="6"/>
+      <c r="B92" s="3"/>
+      <c r="C92" s="3"/>
+      <c r="D92" s="3"/>
+      <c r="E92" s="3"/>
+      <c r="F92" s="3"/>
+      <c r="G92" s="3"/>
+      <c r="H92" s="3"/>
+      <c r="I92" s="3"/>
+      <c r="J92" s="9"/>
+    </row>
+    <row r="93" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A93" s="6"/>
+      <c r="B93" s="3"/>
+      <c r="C93" s="3"/>
+      <c r="D93" s="3"/>
+      <c r="E93" s="3"/>
+      <c r="F93" s="3"/>
+      <c r="G93" s="3"/>
+      <c r="H93" s="3"/>
+      <c r="I93" s="3"/>
+      <c r="J93" s="9"/>
+    </row>
+    <row r="94" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A94" s="6"/>
+      <c r="B94" s="3"/>
+      <c r="C94" s="3"/>
+      <c r="D94" s="3"/>
+      <c r="E94" s="3"/>
+      <c r="F94" s="3"/>
+      <c r="G94" s="3"/>
+      <c r="H94" s="3"/>
+      <c r="I94" s="3"/>
+      <c r="J94" s="9"/>
+    </row>
+    <row r="95" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A95" s="6"/>
+      <c r="B95" s="3"/>
+      <c r="C95" s="3"/>
+      <c r="D95" s="3"/>
+      <c r="E95" s="3"/>
+      <c r="F95" s="3"/>
+      <c r="G95" s="3"/>
+      <c r="H95" s="3"/>
+      <c r="I95" s="3"/>
+      <c r="J95" s="9"/>
+    </row>
+    <row r="96" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A96" s="6"/>
+      <c r="B96" s="3"/>
+      <c r="C96" s="3"/>
+      <c r="D96" s="3"/>
+      <c r="E96" s="3"/>
+      <c r="F96" s="3"/>
+      <c r="G96" s="3"/>
+      <c r="H96" s="3"/>
+      <c r="I96" s="3"/>
+      <c r="J96" s="9"/>
+    </row>
+    <row r="97" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A97" s="6"/>
+      <c r="B97" s="3"/>
+      <c r="C97" s="3"/>
+      <c r="D97" s="3"/>
+      <c r="E97" s="3"/>
+      <c r="F97" s="3"/>
+      <c r="G97" s="3"/>
+      <c r="H97" s="3"/>
+      <c r="I97" s="3"/>
+      <c r="J97" s="9"/>
+    </row>
+    <row r="98" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A98" s="6"/>
+      <c r="B98" s="3"/>
+      <c r="C98" s="3"/>
+      <c r="D98" s="3"/>
+      <c r="E98" s="3"/>
+      <c r="F98" s="3"/>
+      <c r="G98" s="3"/>
+      <c r="H98" s="3"/>
+      <c r="I98" s="3"/>
+      <c r="J98" s="9"/>
+    </row>
+    <row r="99" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A99" s="6"/>
+      <c r="B99" s="3"/>
+      <c r="C99" s="3"/>
+      <c r="D99" s="3"/>
+      <c r="E99" s="3"/>
+      <c r="F99" s="3"/>
+      <c r="G99" s="3"/>
+      <c r="H99" s="3"/>
+      <c r="I99" s="3"/>
+      <c r="J99" s="9"/>
+    </row>
+    <row r="100" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A100" s="6"/>
+      <c r="B100" s="3"/>
+      <c r="C100" s="3"/>
+      <c r="D100" s="3"/>
+      <c r="E100" s="3"/>
+      <c r="F100" s="3"/>
+      <c r="G100" s="3"/>
+      <c r="H100" s="3"/>
+      <c r="I100" s="3"/>
+      <c r="J100" s="9"/>
+    </row>
+    <row r="101" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A101" s="6"/>
+      <c r="B101" s="3"/>
+      <c r="C101" s="3"/>
+      <c r="D101" s="3"/>
+      <c r="E101" s="3"/>
+      <c r="F101" s="3"/>
+      <c r="G101" s="3"/>
+      <c r="H101" s="3"/>
+      <c r="I101" s="3"/>
+      <c r="J101" s="9"/>
+    </row>
+    <row r="102" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A102" s="6"/>
+      <c r="B102" s="3"/>
+      <c r="C102" s="3"/>
+      <c r="D102" s="3"/>
+      <c r="E102" s="3"/>
+      <c r="F102" s="3"/>
+      <c r="G102" s="3"/>
+      <c r="H102" s="3"/>
+      <c r="I102" s="3"/>
+      <c r="J102" s="9"/>
+    </row>
+    <row r="103" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A103" s="6"/>
+      <c r="B103" s="3"/>
+      <c r="C103" s="3"/>
+      <c r="D103" s="3"/>
+      <c r="E103" s="3"/>
+      <c r="F103" s="3"/>
+      <c r="G103" s="3"/>
+      <c r="H103" s="3"/>
+      <c r="I103" s="3"/>
+      <c r="J103" s="9"/>
+    </row>
+    <row r="104" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A104" s="6"/>
+      <c r="B104" s="3"/>
+      <c r="C104" s="3"/>
+      <c r="D104" s="3"/>
+      <c r="E104" s="3"/>
+      <c r="F104" s="3"/>
+      <c r="G104" s="3"/>
+      <c r="H104" s="3"/>
+      <c r="I104" s="3"/>
+      <c r="J104" s="9"/>
+    </row>
+    <row r="105" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A105" s="6"/>
+      <c r="B105" s="3"/>
+      <c r="C105" s="3"/>
+      <c r="D105" s="3"/>
+      <c r="E105" s="3"/>
+      <c r="F105" s="3"/>
+      <c r="G105" s="3"/>
+      <c r="H105" s="3"/>
+      <c r="I105" s="3"/>
+      <c r="J105" s="9"/>
+    </row>
+    <row r="106" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A106" s="6"/>
+      <c r="B106" s="3"/>
+      <c r="C106" s="3"/>
+      <c r="D106" s="3"/>
+      <c r="E106" s="3"/>
+      <c r="F106" s="3"/>
+      <c r="G106" s="3"/>
+      <c r="H106" s="3"/>
+      <c r="I106" s="3"/>
+      <c r="J106" s="9"/>
+    </row>
+    <row r="107" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A107" s="6"/>
+      <c r="B107" s="3"/>
+      <c r="C107" s="3"/>
+      <c r="D107" s="3"/>
+      <c r="E107" s="3"/>
+      <c r="F107" s="3"/>
+      <c r="G107" s="3"/>
+      <c r="H107" s="3"/>
+      <c r="I107" s="3"/>
+      <c r="J107" s="9"/>
+    </row>
+    <row r="108" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A108" s="6"/>
+      <c r="B108" s="3"/>
+      <c r="C108" s="3"/>
+      <c r="D108" s="3"/>
+      <c r="E108" s="3"/>
+      <c r="F108" s="3"/>
+      <c r="G108" s="3"/>
+      <c r="H108" s="3"/>
+      <c r="I108" s="3"/>
+      <c r="J108" s="9"/>
+    </row>
+    <row r="109" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A109" s="6"/>
+      <c r="B109" s="3"/>
+      <c r="C109" s="3"/>
+      <c r="D109" s="3"/>
+      <c r="E109" s="3"/>
+      <c r="F109" s="3"/>
+      <c r="G109" s="3"/>
+      <c r="H109" s="3"/>
+      <c r="I109" s="3"/>
+      <c r="J109" s="9"/>
+    </row>
+    <row r="110" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A110" s="6"/>
+      <c r="B110" s="3"/>
+      <c r="C110" s="3"/>
+      <c r="D110" s="3"/>
+      <c r="E110" s="3"/>
+      <c r="F110" s="3"/>
+      <c r="G110" s="3"/>
+      <c r="H110" s="3"/>
+      <c r="I110" s="3"/>
+      <c r="J110" s="9"/>
+    </row>
+    <row r="111" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A111" s="6"/>
+      <c r="B111" s="3"/>
+      <c r="C111" s="3"/>
+      <c r="D111" s="3"/>
+      <c r="E111" s="3"/>
+      <c r="F111" s="3"/>
+      <c r="G111" s="3"/>
+      <c r="H111" s="3"/>
+      <c r="I111" s="3"/>
+      <c r="J111" s="9"/>
+    </row>
+    <row r="112" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A112" s="6"/>
+      <c r="B112" s="3"/>
+      <c r="C112" s="3"/>
+      <c r="D112" s="3"/>
+      <c r="E112" s="3"/>
+      <c r="F112" s="3"/>
+      <c r="G112" s="3"/>
+      <c r="H112" s="3"/>
+      <c r="I112" s="3"/>
+      <c r="J112" s="9"/>
+    </row>
+    <row r="113" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A113" s="6"/>
+      <c r="B113" s="3"/>
+      <c r="C113" s="3"/>
+      <c r="D113" s="3"/>
+      <c r="E113" s="3"/>
+      <c r="F113" s="3"/>
+      <c r="G113" s="3"/>
+      <c r="H113" s="3"/>
+      <c r="I113" s="3"/>
+      <c r="J113" s="9"/>
+    </row>
+    <row r="114" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A114" s="6"/>
+      <c r="B114" s="3"/>
+      <c r="C114" s="3"/>
+      <c r="D114" s="3"/>
+      <c r="E114" s="3"/>
+      <c r="F114" s="3"/>
+      <c r="G114" s="3"/>
+      <c r="H114" s="3"/>
+      <c r="I114" s="3"/>
+      <c r="J114" s="9"/>
+    </row>
+    <row r="115" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A115" s="6"/>
+      <c r="B115" s="3"/>
+      <c r="C115" s="3"/>
+      <c r="D115" s="3"/>
+      <c r="E115" s="3"/>
+      <c r="F115" s="3"/>
+      <c r="G115" s="3"/>
+      <c r="H115" s="3"/>
+      <c r="I115" s="3"/>
+      <c r="J115" s="9"/>
+    </row>
+    <row r="116" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A116" s="6"/>
+      <c r="B116" s="3"/>
+      <c r="C116" s="3"/>
+      <c r="D116" s="3"/>
+      <c r="E116" s="3"/>
+      <c r="F116" s="3"/>
+      <c r="G116" s="3"/>
+      <c r="H116" s="3"/>
+      <c r="I116" s="3"/>
+      <c r="J116" s="9"/>
+    </row>
+    <row r="117" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A117" s="6"/>
+      <c r="B117" s="3"/>
+      <c r="C117" s="3"/>
+      <c r="D117" s="3"/>
+      <c r="E117" s="3"/>
+      <c r="F117" s="3"/>
+      <c r="G117" s="3"/>
+      <c r="H117" s="3"/>
+      <c r="I117" s="3"/>
+      <c r="J117" s="9"/>
+    </row>
+    <row r="118" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A118" s="6"/>
+      <c r="B118" s="3"/>
+      <c r="C118" s="3"/>
+      <c r="D118" s="3"/>
+      <c r="E118" s="3"/>
+      <c r="F118" s="3"/>
+      <c r="G118" s="3"/>
+      <c r="H118" s="3"/>
+      <c r="I118" s="3"/>
+      <c r="J118" s="9"/>
+    </row>
+    <row r="119" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A119" s="6"/>
+      <c r="B119" s="3"/>
+      <c r="C119" s="3"/>
+      <c r="D119" s="3"/>
+      <c r="E119" s="3"/>
+      <c r="F119" s="3"/>
+      <c r="G119" s="3"/>
+      <c r="H119" s="3"/>
+      <c r="I119" s="3"/>
+      <c r="J119" s="9"/>
+    </row>
+    <row r="120" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A120" s="6"/>
+      <c r="B120" s="3"/>
+      <c r="C120" s="3"/>
+      <c r="D120" s="3"/>
+      <c r="E120" s="3"/>
+      <c r="F120" s="3"/>
+      <c r="G120" s="3"/>
+      <c r="H120" s="3"/>
+      <c r="I120" s="3"/>
+      <c r="J120" s="9"/>
+    </row>
+    <row r="121" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A121" s="6"/>
+      <c r="B121" s="3"/>
+      <c r="C121" s="3"/>
+      <c r="D121" s="3"/>
+      <c r="E121" s="3"/>
+      <c r="F121" s="3"/>
+      <c r="G121" s="3"/>
+      <c r="H121" s="3"/>
+      <c r="I121" s="3"/>
+      <c r="J121" s="9"/>
+    </row>
+    <row r="122" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A122" s="6"/>
+      <c r="B122" s="3"/>
+      <c r="C122" s="3"/>
+      <c r="D122" s="3"/>
+      <c r="E122" s="3"/>
+      <c r="F122" s="3"/>
+      <c r="G122" s="3"/>
+      <c r="H122" s="3"/>
+      <c r="I122" s="3"/>
+      <c r="J122" s="9"/>
+    </row>
+    <row r="123" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A123" s="6"/>
+      <c r="B123" s="3"/>
+      <c r="C123" s="3"/>
+      <c r="D123" s="3"/>
+      <c r="E123" s="3"/>
+      <c r="F123" s="3"/>
+      <c r="G123" s="3"/>
+      <c r="H123" s="3"/>
+      <c r="I123" s="3"/>
+      <c r="J123" s="9"/>
+    </row>
+    <row r="124" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A124" s="6"/>
+      <c r="B124" s="3"/>
+      <c r="C124" s="3"/>
+      <c r="D124" s="3"/>
+      <c r="E124" s="3"/>
+      <c r="F124" s="3"/>
+      <c r="G124" s="3"/>
+      <c r="H124" s="3"/>
+      <c r="I124" s="3"/>
+      <c r="J124" s="9"/>
+    </row>
+    <row r="125" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A125" s="6"/>
+      <c r="B125" s="3"/>
+      <c r="C125" s="3"/>
+      <c r="D125" s="3"/>
+      <c r="E125" s="3"/>
+      <c r="F125" s="3"/>
+      <c r="G125" s="3"/>
+      <c r="H125" s="3"/>
+      <c r="I125" s="3"/>
+      <c r="J125" s="9"/>
+    </row>
+    <row r="126" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A126" s="6"/>
+      <c r="B126" s="3"/>
+      <c r="C126" s="3"/>
+      <c r="D126" s="3"/>
+      <c r="E126" s="3"/>
+      <c r="F126" s="3"/>
+      <c r="G126" s="3"/>
+      <c r="H126" s="3"/>
+      <c r="I126" s="3"/>
+      <c r="J126" s="9"/>
+    </row>
+    <row r="127" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A127" s="6"/>
+      <c r="B127" s="3"/>
+      <c r="C127" s="3"/>
+      <c r="D127" s="3"/>
+      <c r="E127" s="3"/>
+      <c r="F127" s="3"/>
+      <c r="G127" s="3"/>
+      <c r="H127" s="3"/>
+      <c r="I127" s="3"/>
+      <c r="J127" s="9"/>
+    </row>
+    <row r="128" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A128" s="6"/>
+      <c r="B128" s="3"/>
+      <c r="C128" s="3"/>
+      <c r="D128" s="3"/>
+      <c r="E128" s="3"/>
+      <c r="F128" s="3"/>
+      <c r="G128" s="3"/>
+      <c r="H128" s="3"/>
+      <c r="I128" s="3"/>
+      <c r="J128" s="9"/>
+    </row>
+    <row r="129" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A129" s="6"/>
+      <c r="B129" s="3"/>
+      <c r="C129" s="3"/>
+      <c r="D129" s="3"/>
+      <c r="E129" s="3"/>
+      <c r="F129" s="3"/>
+      <c r="G129" s="3"/>
+      <c r="H129" s="3"/>
+      <c r="I129" s="3"/>
+      <c r="J129" s="9"/>
+    </row>
+    <row r="130" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A130" s="6"/>
+      <c r="B130" s="3"/>
+      <c r="C130" s="3"/>
+      <c r="D130" s="3"/>
+      <c r="E130" s="3"/>
+      <c r="F130" s="3"/>
+      <c r="G130" s="3"/>
+      <c r="H130" s="3"/>
+      <c r="I130" s="3"/>
+      <c r="J130" s="9"/>
+    </row>
+    <row r="131" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A131" s="6"/>
+      <c r="B131" s="3"/>
+      <c r="C131" s="3"/>
+      <c r="D131" s="3"/>
+      <c r="E131" s="3"/>
+      <c r="F131" s="3"/>
+      <c r="G131" s="3"/>
+      <c r="H131" s="3"/>
+      <c r="I131" s="3"/>
+      <c r="J131" s="9"/>
+    </row>
+    <row r="132" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A132" s="6"/>
+      <c r="B132" s="3"/>
+      <c r="C132" s="3"/>
+      <c r="D132" s="3"/>
+      <c r="E132" s="3"/>
+      <c r="F132" s="3"/>
+      <c r="G132" s="3"/>
+      <c r="H132" s="3"/>
+      <c r="I132" s="3"/>
+      <c r="J132" s="9"/>
+    </row>
+    <row r="133" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A133" s="6"/>
+      <c r="B133" s="3"/>
+      <c r="C133" s="3"/>
+      <c r="D133" s="3"/>
+      <c r="E133" s="3"/>
+      <c r="F133" s="3"/>
+      <c r="G133" s="3"/>
+      <c r="H133" s="3"/>
+      <c r="I133" s="3"/>
+      <c r="J133" s="9"/>
+    </row>
+    <row r="134" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A134" s="6"/>
+      <c r="B134" s="3"/>
+      <c r="C134" s="3"/>
+      <c r="D134" s="3"/>
+      <c r="E134" s="3"/>
+      <c r="F134" s="3"/>
+      <c r="G134" s="3"/>
+      <c r="H134" s="3"/>
+      <c r="I134" s="3"/>
+      <c r="J134" s="9"/>
+    </row>
+    <row r="135" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A135" s="6"/>
+      <c r="B135" s="3"/>
+      <c r="C135" s="3"/>
+      <c r="D135" s="3"/>
+      <c r="E135" s="3"/>
+      <c r="F135" s="3"/>
+      <c r="G135" s="3"/>
+      <c r="H135" s="3"/>
+      <c r="I135" s="3"/>
+      <c r="J135" s="9"/>
+    </row>
+    <row r="136" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A136" s="6"/>
+      <c r="B136" s="3"/>
+      <c r="C136" s="3"/>
+      <c r="D136" s="3"/>
+      <c r="E136" s="3"/>
+      <c r="F136" s="3"/>
+      <c r="G136" s="3"/>
+      <c r="H136" s="3"/>
+      <c r="I136" s="3"/>
+      <c r="J136" s="9"/>
+    </row>
+    <row r="137" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A137" s="6"/>
+      <c r="B137" s="3"/>
+      <c r="C137" s="3"/>
+      <c r="D137" s="3"/>
+      <c r="E137" s="3"/>
+      <c r="F137" s="3"/>
+      <c r="G137" s="3"/>
+      <c r="H137" s="3"/>
+      <c r="I137" s="3"/>
+      <c r="J137" s="9"/>
+    </row>
+    <row r="138" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A138" s="6"/>
+      <c r="B138" s="3"/>
+      <c r="C138" s="3"/>
+      <c r="D138" s="3"/>
+      <c r="E138" s="3"/>
+      <c r="F138" s="3"/>
+      <c r="G138" s="3"/>
+      <c r="H138" s="3"/>
+      <c r="I138" s="3"/>
+      <c r="J138" s="9"/>
+    </row>
+    <row r="139" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A139" s="6"/>
+      <c r="B139" s="3"/>
+      <c r="C139" s="3"/>
+      <c r="D139" s="3"/>
+      <c r="E139" s="3"/>
+      <c r="F139" s="3"/>
+      <c r="G139" s="3"/>
+      <c r="H139" s="3"/>
+      <c r="I139" s="3"/>
+      <c r="J139" s="9"/>
+    </row>
+    <row r="140" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A140" s="6"/>
+      <c r="B140" s="3"/>
+      <c r="C140" s="3"/>
+      <c r="D140" s="3"/>
+      <c r="E140" s="3"/>
+      <c r="F140" s="3"/>
+      <c r="G140" s="3"/>
+      <c r="H140" s="3"/>
+      <c r="I140" s="3"/>
+      <c r="J140" s="9"/>
+    </row>
+    <row r="141" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A141" s="6"/>
+      <c r="B141" s="3"/>
+      <c r="C141" s="3"/>
+      <c r="D141" s="3"/>
+      <c r="E141" s="3"/>
+      <c r="F141" s="3"/>
+      <c r="G141" s="3"/>
+      <c r="H141" s="3"/>
+      <c r="I141" s="3"/>
+      <c r="J141" s="9"/>
+    </row>
+    <row r="142" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A142" s="6"/>
+      <c r="B142" s="3"/>
+      <c r="C142" s="3"/>
+      <c r="D142" s="3"/>
+      <c r="E142" s="3"/>
+      <c r="F142" s="3"/>
+      <c r="G142" s="3"/>
+      <c r="H142" s="3"/>
+      <c r="I142" s="3"/>
+      <c r="J142" s="9"/>
+    </row>
+    <row r="143" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A143" s="6"/>
+      <c r="B143" s="3"/>
+      <c r="C143" s="3"/>
+      <c r="D143" s="3"/>
+      <c r="E143" s="3"/>
+      <c r="F143" s="3"/>
+      <c r="G143" s="3"/>
+      <c r="H143" s="3"/>
+      <c r="I143" s="3"/>
+      <c r="J143" s="9"/>
+    </row>
+    <row r="144" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A144" s="6"/>
+      <c r="B144" s="3"/>
+      <c r="C144" s="3"/>
+      <c r="D144" s="3"/>
+      <c r="E144" s="3"/>
+      <c r="F144" s="3"/>
+      <c r="G144" s="3"/>
+      <c r="H144" s="3"/>
+      <c r="I144" s="3"/>
+      <c r="J144" s="9"/>
+    </row>
+    <row r="145" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A145" s="6"/>
+      <c r="B145" s="3"/>
+      <c r="C145" s="3"/>
+      <c r="D145" s="3"/>
+      <c r="E145" s="3"/>
+      <c r="F145" s="3"/>
+      <c r="G145" s="3"/>
+      <c r="H145" s="3"/>
+      <c r="I145" s="3"/>
+      <c r="J145" s="9"/>
+    </row>
+    <row r="146" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A146" s="6"/>
+      <c r="B146" s="3"/>
+      <c r="C146" s="3"/>
+      <c r="D146" s="3"/>
+      <c r="E146" s="3"/>
+      <c r="F146" s="3"/>
+      <c r="G146" s="3"/>
+      <c r="H146" s="3"/>
+      <c r="I146" s="3"/>
+      <c r="J146" s="9"/>
+    </row>
+    <row r="147" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A147" s="6"/>
+      <c r="B147" s="3"/>
+      <c r="C147" s="3"/>
+      <c r="D147" s="3"/>
+      <c r="E147" s="3"/>
+      <c r="F147" s="3"/>
+      <c r="G147" s="3"/>
+      <c r="H147" s="3"/>
+      <c r="I147" s="3"/>
+      <c r="J147" s="9"/>
+    </row>
+    <row r="148" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A148" s="6"/>
+      <c r="B148" s="3"/>
+      <c r="C148" s="3"/>
+      <c r="D148" s="3"/>
+      <c r="E148" s="3"/>
+      <c r="F148" s="3"/>
+      <c r="G148" s="3"/>
+      <c r="H148" s="3"/>
+      <c r="I148" s="3"/>
+      <c r="J148" s="9"/>
+    </row>
+    <row r="149" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A149" s="6"/>
+      <c r="B149" s="3"/>
+      <c r="C149" s="3"/>
+      <c r="D149" s="3"/>
+      <c r="E149" s="3"/>
+      <c r="F149" s="3"/>
+      <c r="G149" s="3"/>
+      <c r="H149" s="3"/>
+      <c r="I149" s="3"/>
+      <c r="J149" s="9"/>
+    </row>
+    <row r="150" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A150" s="6"/>
+      <c r="B150" s="3"/>
+      <c r="C150" s="3"/>
+      <c r="D150" s="3"/>
+      <c r="E150" s="3"/>
+      <c r="F150" s="3"/>
+      <c r="G150" s="3"/>
+      <c r="H150" s="3"/>
+      <c r="I150" s="3"/>
+      <c r="J150" s="9"/>
+    </row>
+    <row r="151" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A151" s="6"/>
+      <c r="B151" s="3"/>
+      <c r="C151" s="3"/>
+      <c r="D151" s="3"/>
+      <c r="E151" s="3"/>
+      <c r="F151" s="3"/>
+      <c r="G151" s="3"/>
+      <c r="H151" s="3"/>
+      <c r="I151" s="3"/>
+      <c r="J151" s="9"/>
+    </row>
+    <row r="152" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A152" s="6"/>
+      <c r="B152" s="3"/>
+      <c r="C152" s="3"/>
+      <c r="D152" s="3"/>
+      <c r="E152" s="3"/>
+      <c r="F152" s="3"/>
+      <c r="G152" s="3"/>
+      <c r="H152" s="3"/>
+      <c r="I152" s="3"/>
+      <c r="J152" s="9"/>
+    </row>
+    <row r="153" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A153" s="6"/>
+      <c r="B153" s="3"/>
+      <c r="C153" s="3"/>
+      <c r="D153" s="3"/>
+      <c r="E153" s="3"/>
+      <c r="F153" s="3"/>
+      <c r="G153" s="3"/>
+      <c r="H153" s="3"/>
+      <c r="I153" s="3"/>
+      <c r="J153" s="9"/>
+    </row>
+    <row r="154" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A154" s="6"/>
+      <c r="B154" s="3"/>
+      <c r="C154" s="3"/>
+      <c r="D154" s="3"/>
+      <c r="E154" s="3"/>
+      <c r="F154" s="3"/>
+      <c r="G154" s="3"/>
+      <c r="H154" s="3"/>
+      <c r="I154" s="3"/>
+      <c r="J154" s="9"/>
+    </row>
+    <row r="155" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A155" s="6"/>
+      <c r="B155" s="3"/>
+      <c r="C155" s="3"/>
+      <c r="D155" s="3"/>
+      <c r="E155" s="3"/>
+      <c r="F155" s="3"/>
+      <c r="G155" s="3"/>
+      <c r="H155" s="3"/>
+      <c r="I155" s="3"/>
+      <c r="J155" s="9"/>
+    </row>
+    <row r="156" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A156" s="6"/>
+      <c r="B156" s="3"/>
+      <c r="C156" s="3"/>
+      <c r="D156" s="3"/>
+      <c r="E156" s="3"/>
+      <c r="F156" s="3"/>
+      <c r="G156" s="3"/>
+      <c r="H156" s="3"/>
+      <c r="I156" s="3"/>
+      <c r="J156" s="9"/>
+    </row>
+    <row r="157" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A157" s="6"/>
+      <c r="B157" s="3"/>
+      <c r="C157" s="3"/>
+      <c r="D157" s="3"/>
+      <c r="E157" s="3"/>
+      <c r="F157" s="3"/>
+      <c r="G157" s="3"/>
+      <c r="H157" s="3"/>
+      <c r="I157" s="3"/>
+      <c r="J157" s="9"/>
+    </row>
+    <row r="158" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A158" s="6"/>
+      <c r="B158" s="3"/>
+      <c r="C158" s="3"/>
+      <c r="D158" s="3"/>
+      <c r="E158" s="3"/>
+      <c r="F158" s="3"/>
+      <c r="G158" s="3"/>
+      <c r="H158" s="3"/>
+      <c r="I158" s="3"/>
+      <c r="J158" s="9"/>
+    </row>
+    <row r="159" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A159" s="6"/>
+      <c r="B159" s="3"/>
+      <c r="C159" s="3"/>
+      <c r="D159" s="3"/>
+      <c r="E159" s="3"/>
+      <c r="F159" s="3"/>
+      <c r="G159" s="3"/>
+      <c r="H159" s="3"/>
+      <c r="I159" s="3"/>
+      <c r="J159" s="9"/>
+    </row>
+    <row r="160" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A160" s="6"/>
+      <c r="B160" s="3"/>
+      <c r="C160" s="3"/>
+      <c r="D160" s="3"/>
+      <c r="E160" s="3"/>
+      <c r="F160" s="3"/>
+      <c r="G160" s="3"/>
+      <c r="H160" s="3"/>
+      <c r="I160" s="3"/>
+      <c r="J160" s="9"/>
+    </row>
+    <row r="161" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A161" s="6"/>
+      <c r="B161" s="3"/>
+      <c r="C161" s="3"/>
+      <c r="D161" s="3"/>
+      <c r="E161" s="3"/>
+      <c r="F161" s="3"/>
+      <c r="G161" s="3"/>
+      <c r="H161" s="3"/>
+      <c r="I161" s="3"/>
+      <c r="J161" s="9"/>
+    </row>
+    <row r="162" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A162" s="6"/>
+      <c r="B162" s="3"/>
+      <c r="C162" s="3"/>
+      <c r="D162" s="3"/>
+      <c r="E162" s="3"/>
+      <c r="F162" s="3"/>
+      <c r="G162" s="3"/>
+      <c r="H162" s="3"/>
+      <c r="I162" s="3"/>
+      <c r="J162" s="9"/>
+    </row>
+    <row r="163" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A163" s="6"/>
+      <c r="B163" s="3"/>
+      <c r="C163" s="3"/>
+      <c r="D163" s="3"/>
+      <c r="E163" s="3"/>
+      <c r="F163" s="3"/>
+      <c r="G163" s="3"/>
+      <c r="H163" s="3"/>
+      <c r="I163" s="3"/>
+      <c r="J163" s="9"/>
+    </row>
+    <row r="164" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A164" s="6"/>
+      <c r="B164" s="3"/>
+      <c r="C164" s="3"/>
+      <c r="D164" s="3"/>
+      <c r="E164" s="3"/>
+      <c r="F164" s="3"/>
+      <c r="G164" s="3"/>
+      <c r="H164" s="3"/>
+      <c r="I164" s="3"/>
+      <c r="J164" s="9"/>
+    </row>
+    <row r="165" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A165" s="6"/>
+      <c r="B165" s="3"/>
+      <c r="C165" s="3"/>
+      <c r="D165" s="3"/>
+      <c r="E165" s="3"/>
+      <c r="F165" s="3"/>
+      <c r="G165" s="3"/>
+      <c r="H165" s="3"/>
+      <c r="I165" s="3"/>
+      <c r="J165" s="9"/>
+    </row>
+    <row r="166" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A166" s="6"/>
+      <c r="B166" s="3"/>
+      <c r="C166" s="3"/>
+      <c r="D166" s="3"/>
+      <c r="E166" s="3"/>
+      <c r="F166" s="3"/>
+      <c r="G166" s="3"/>
+      <c r="H166" s="3"/>
+      <c r="I166" s="3"/>
+      <c r="J166" s="9"/>
+    </row>
+    <row r="167" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A167" s="6"/>
+      <c r="B167" s="3"/>
+      <c r="C167" s="3"/>
+      <c r="D167" s="3"/>
+      <c r="E167" s="3"/>
+      <c r="F167" s="3"/>
+      <c r="G167" s="3"/>
+      <c r="H167" s="3"/>
+      <c r="I167" s="3"/>
+      <c r="J167" s="9"/>
+    </row>
+    <row r="168" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A168" s="6"/>
+      <c r="B168" s="3"/>
+      <c r="C168" s="3"/>
+      <c r="D168" s="3"/>
+      <c r="E168" s="3"/>
+      <c r="F168" s="3"/>
+      <c r="G168" s="3"/>
+      <c r="H168" s="3"/>
+      <c r="I168" s="3"/>
+      <c r="J168" s="9"/>
+    </row>
+    <row r="169" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A169" s="6"/>
+      <c r="B169" s="3"/>
+      <c r="C169" s="3"/>
+      <c r="D169" s="3"/>
+      <c r="E169" s="3"/>
+      <c r="F169" s="3"/>
+      <c r="G169" s="3"/>
+      <c r="H169" s="3"/>
+      <c r="I169" s="3"/>
+      <c r="J169" s="9"/>
+    </row>
+    <row r="170" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A170" s="6"/>
+      <c r="B170" s="3"/>
+      <c r="C170" s="3"/>
+      <c r="D170" s="3"/>
+      <c r="E170" s="3"/>
+      <c r="F170" s="3"/>
+      <c r="G170" s="3"/>
+      <c r="H170" s="3"/>
+      <c r="I170" s="3"/>
+      <c r="J170" s="9"/>
+    </row>
+    <row r="171" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A171" s="6"/>
+      <c r="B171" s="3"/>
+      <c r="C171" s="3"/>
+      <c r="D171" s="3"/>
+      <c r="E171" s="3"/>
+      <c r="F171" s="3"/>
+      <c r="G171" s="3"/>
+      <c r="H171" s="3"/>
+      <c r="I171" s="3"/>
+      <c r="J171" s="9"/>
+    </row>
+    <row r="172" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A172" s="6"/>
+      <c r="B172" s="3"/>
+      <c r="C172" s="3"/>
+      <c r="D172" s="3"/>
+      <c r="E172" s="3"/>
+      <c r="F172" s="3"/>
+      <c r="G172" s="3"/>
+      <c r="H172" s="3"/>
+      <c r="I172" s="3"/>
+      <c r="J172" s="9"/>
+    </row>
+    <row r="173" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A173" s="6"/>
+      <c r="B173" s="3"/>
+      <c r="C173" s="3"/>
+      <c r="D173" s="3"/>
+      <c r="E173" s="3"/>
+      <c r="F173" s="3"/>
+      <c r="G173" s="3"/>
+      <c r="H173" s="3"/>
+      <c r="I173" s="3"/>
+      <c r="J173" s="9"/>
+    </row>
+    <row r="174" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A174" s="6"/>
+      <c r="B174" s="3"/>
+      <c r="C174" s="3"/>
+      <c r="D174" s="3"/>
+      <c r="E174" s="3"/>
+      <c r="F174" s="3"/>
+      <c r="G174" s="3"/>
+      <c r="H174" s="3"/>
+      <c r="I174" s="3"/>
+      <c r="J174" s="9"/>
+    </row>
+    <row r="175" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A175" s="6"/>
+      <c r="B175" s="3"/>
+      <c r="C175" s="3"/>
+      <c r="D175" s="3"/>
+      <c r="E175" s="3"/>
+      <c r="F175" s="3"/>
+      <c r="G175" s="3"/>
+      <c r="H175" s="3"/>
+      <c r="I175" s="3"/>
+      <c r="J175" s="9"/>
+    </row>
+    <row r="176" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A176" s="6"/>
+      <c r="B176" s="3"/>
+      <c r="C176" s="3"/>
+      <c r="D176" s="3"/>
+      <c r="E176" s="3"/>
+      <c r="F176" s="3"/>
+      <c r="G176" s="3"/>
+      <c r="H176" s="3"/>
+      <c r="I176" s="3"/>
+      <c r="J176" s="9"/>
+    </row>
+    <row r="177" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A177" s="6"/>
+      <c r="B177" s="3"/>
+      <c r="C177" s="3"/>
+      <c r="D177" s="3"/>
+      <c r="E177" s="3"/>
+      <c r="F177" s="3"/>
+      <c r="G177" s="3"/>
+      <c r="H177" s="3"/>
+      <c r="I177" s="3"/>
+      <c r="J177" s="9"/>
+    </row>
+    <row r="178" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A178" s="6"/>
+      <c r="B178" s="3"/>
+      <c r="C178" s="3"/>
+      <c r="D178" s="3"/>
+      <c r="E178" s="3"/>
+      <c r="F178" s="3"/>
+      <c r="G178" s="3"/>
+      <c r="H178" s="3"/>
+      <c r="I178" s="3"/>
+      <c r="J178" s="9"/>
+    </row>
+    <row r="179" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A179" s="6"/>
+      <c r="B179" s="3"/>
+      <c r="C179" s="3"/>
+      <c r="D179" s="3"/>
+      <c r="E179" s="3"/>
+      <c r="F179" s="3"/>
+      <c r="G179" s="3"/>
+      <c r="H179" s="3"/>
+      <c r="I179" s="3"/>
+      <c r="J179" s="9"/>
+    </row>
+    <row r="180" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A180" s="6"/>
+      <c r="B180" s="3"/>
+      <c r="C180" s="3"/>
+      <c r="D180" s="3"/>
+      <c r="E180" s="3"/>
+      <c r="F180" s="3"/>
+      <c r="G180" s="3"/>
+      <c r="H180" s="3"/>
+      <c r="I180" s="3"/>
+      <c r="J180" s="9"/>
+    </row>
+    <row r="181" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A181" s="6"/>
+      <c r="B181" s="3"/>
+      <c r="C181" s="3"/>
+      <c r="D181" s="3"/>
+      <c r="E181" s="3"/>
+      <c r="F181" s="3"/>
+      <c r="G181" s="3"/>
+      <c r="H181" s="3"/>
+      <c r="I181" s="3"/>
+      <c r="J181" s="9"/>
+    </row>
+    <row r="182" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A182" s="6"/>
+      <c r="B182" s="3"/>
+      <c r="C182" s="3"/>
+      <c r="D182" s="3"/>
+      <c r="E182" s="3"/>
+      <c r="F182" s="3"/>
+      <c r="G182" s="3"/>
+      <c r="H182" s="3"/>
+      <c r="I182" s="3"/>
+      <c r="J182" s="9"/>
+    </row>
+    <row r="183" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A183" s="6"/>
+      <c r="B183" s="3"/>
+      <c r="C183" s="3"/>
+      <c r="D183" s="3"/>
+      <c r="E183" s="3"/>
+      <c r="F183" s="3"/>
+      <c r="G183" s="3"/>
+      <c r="H183" s="3"/>
+      <c r="I183" s="3"/>
+      <c r="J183" s="9"/>
+    </row>
+    <row r="184" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A184" s="6"/>
+      <c r="B184" s="3"/>
+      <c r="C184" s="3"/>
+      <c r="D184" s="3"/>
+      <c r="E184" s="3"/>
+      <c r="F184" s="3"/>
+      <c r="G184" s="3"/>
+      <c r="H184" s="3"/>
+      <c r="I184" s="3"/>
+      <c r="J184" s="9"/>
+    </row>
+    <row r="185" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A185" s="6"/>
+      <c r="B185" s="3"/>
+      <c r="C185" s="3"/>
+      <c r="D185" s="3"/>
+      <c r="E185" s="3"/>
+      <c r="F185" s="3"/>
+      <c r="G185" s="3"/>
+      <c r="H185" s="3"/>
+      <c r="I185" s="3"/>
+      <c r="J185" s="9"/>
+    </row>
+    <row r="186" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A186" s="6"/>
+      <c r="B186" s="3"/>
+      <c r="C186" s="3"/>
+      <c r="D186" s="3"/>
+      <c r="E186" s="3"/>
+      <c r="F186" s="3"/>
+      <c r="G186" s="3"/>
+      <c r="H186" s="3"/>
+      <c r="I186" s="3"/>
+      <c r="J186" s="9"/>
+    </row>
+    <row r="187" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A187" s="6"/>
+      <c r="B187" s="3"/>
+      <c r="C187" s="3"/>
+      <c r="D187" s="3"/>
+      <c r="E187" s="3"/>
+      <c r="F187" s="3"/>
+      <c r="G187" s="3"/>
+      <c r="H187" s="3"/>
+      <c r="I187" s="3"/>
+      <c r="J187" s="9"/>
+    </row>
+    <row r="188" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A188" s="6"/>
+      <c r="B188" s="3"/>
+      <c r="C188" s="3"/>
+      <c r="D188" s="3"/>
+      <c r="E188" s="3"/>
+      <c r="F188" s="3"/>
+      <c r="G188" s="3"/>
+      <c r="H188" s="3"/>
+      <c r="I188" s="3"/>
+      <c r="J188" s="9"/>
+    </row>
+    <row r="189" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A189" s="6"/>
+      <c r="B189" s="3"/>
+      <c r="C189" s="3"/>
+      <c r="D189" s="3"/>
+      <c r="E189" s="3"/>
+      <c r="F189" s="3"/>
+      <c r="G189" s="3"/>
+      <c r="H189" s="3"/>
+      <c r="I189" s="3"/>
+      <c r="J189" s="9"/>
+    </row>
+    <row r="190" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A190" s="6"/>
+      <c r="B190" s="3"/>
+      <c r="C190" s="3"/>
+      <c r="D190" s="3"/>
+      <c r="E190" s="3"/>
+      <c r="F190" s="3"/>
+      <c r="G190" s="3"/>
+      <c r="H190" s="3"/>
+      <c r="I190" s="3"/>
+      <c r="J190" s="9"/>
+    </row>
+    <row r="191" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A191" s="6"/>
+      <c r="B191" s="3"/>
+      <c r="C191" s="3"/>
+      <c r="D191" s="3"/>
+      <c r="E191" s="3"/>
+      <c r="F191" s="3"/>
+      <c r="G191" s="3"/>
+      <c r="H191" s="3"/>
+      <c r="I191" s="3"/>
+      <c r="J191" s="9"/>
+    </row>
+    <row r="192" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A192" s="6"/>
+      <c r="B192" s="3"/>
+      <c r="C192" s="3"/>
+      <c r="D192" s="3"/>
+      <c r="E192" s="3"/>
+      <c r="F192" s="3"/>
+      <c r="G192" s="3"/>
+      <c r="H192" s="3"/>
+      <c r="I192" s="3"/>
+      <c r="J192" s="9"/>
+    </row>
+    <row r="193" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A193" s="6"/>
+      <c r="B193" s="3"/>
+      <c r="C193" s="3"/>
+      <c r="D193" s="3"/>
+      <c r="E193" s="3"/>
+      <c r="F193" s="3"/>
+      <c r="G193" s="3"/>
+      <c r="H193" s="3"/>
+      <c r="I193" s="3"/>
+      <c r="J193" s="9"/>
+    </row>
+    <row r="194" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A194" s="6"/>
+      <c r="B194" s="3"/>
+      <c r="C194" s="3"/>
+      <c r="D194" s="3"/>
+      <c r="E194" s="3"/>
+      <c r="F194" s="3"/>
+      <c r="G194" s="3"/>
+      <c r="H194" s="3"/>
+      <c r="I194" s="3"/>
+      <c r="J194" s="9"/>
+    </row>
+    <row r="195" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A195" s="6"/>
+      <c r="B195" s="3"/>
+      <c r="C195" s="3"/>
+      <c r="D195" s="3"/>
+      <c r="E195" s="3"/>
+      <c r="F195" s="3"/>
+      <c r="G195" s="3"/>
+      <c r="H195" s="3"/>
+      <c r="I195" s="3"/>
+      <c r="J195" s="9"/>
+    </row>
+    <row r="196" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A196" s="6"/>
+      <c r="B196" s="3"/>
+      <c r="C196" s="3"/>
+      <c r="D196" s="3"/>
+      <c r="E196" s="3"/>
+      <c r="F196" s="3"/>
+      <c r="G196" s="3"/>
+      <c r="H196" s="3"/>
+      <c r="I196" s="3"/>
+      <c r="J196" s="9"/>
+    </row>
+    <row r="197" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A197" s="6"/>
+      <c r="B197" s="3"/>
+      <c r="C197" s="3"/>
+      <c r="D197" s="3"/>
+      <c r="E197" s="3"/>
+      <c r="F197" s="3"/>
+      <c r="G197" s="3"/>
+      <c r="H197" s="3"/>
+      <c r="I197" s="3"/>
+      <c r="J197" s="9"/>
+    </row>
+    <row r="198" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A198" s="6"/>
+      <c r="B198" s="3"/>
+      <c r="C198" s="3"/>
+      <c r="D198" s="3"/>
+      <c r="E198" s="3"/>
+      <c r="F198" s="3"/>
+      <c r="G198" s="3"/>
+      <c r="H198" s="3"/>
+      <c r="I198" s="3"/>
+      <c r="J198" s="9"/>
+    </row>
+    <row r="199" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A199" s="6"/>
+      <c r="B199" s="3"/>
+      <c r="C199" s="3"/>
+      <c r="D199" s="3"/>
+      <c r="E199" s="3"/>
+      <c r="F199" s="3"/>
+      <c r="G199" s="3"/>
+      <c r="H199" s="3"/>
+      <c r="I199" s="3"/>
+      <c r="J199" s="9"/>
+    </row>
+    <row r="200" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A200" s="10"/>
+      <c r="B200" s="11"/>
+      <c r="C200" s="11"/>
+      <c r="D200" s="11"/>
+      <c r="E200" s="11"/>
+      <c r="F200" s="11"/>
+      <c r="G200" s="11"/>
+      <c r="H200" s="11"/>
+      <c r="I200" s="11"/>
+      <c r="J200" s="12"/>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="A1:A2 F2:J3 H4:J7 F12:J19 B2:E7 F4:F7 B8:J11">
+    <cfRule type="expression" dxfId="18" priority="4">
+      <formula>MOD(ROW(),2)=0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B1 D1:J1">
+    <cfRule type="expression" dxfId="17" priority="5">
+      <formula>MOD(ROW(),2)=0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B12:D13">
+    <cfRule type="expression" dxfId="16" priority="2">
+      <formula>MOD(ROW(),2)=0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E12:E15">
+    <cfRule type="expression" dxfId="15" priority="1">
+      <formula>MOD(ROW(),2)=0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E20:J21 A22:J200">
+    <cfRule type="expression" dxfId="14" priority="6">
+      <formula>MOD(ROW(),2)=0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G4:G7">
+    <cfRule type="expression" dxfId="13" priority="3">
+      <formula>MOD(ROW(),2)=0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FFE7585E-75AB-684A-AA88-D151314EB3D5}">
   <dimension ref="A1:J197"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="3" max="3" width="16.5" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="18" x14ac:dyDescent="0.25">
       <c r="A1" s="25">
         <v>1</v>
       </c>
-      <c r="B1" s="18" t="s">
+      <c r="B1" s="23" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="18" t="s">
+      <c r="C1" s="23" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="18" t="s">
+      <c r="D1" s="23" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="18" t="s">
+      <c r="E1" s="23" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="26" t="s">
+      <c r="F1" s="34" t="s">
         <v>31</v>
       </c>
-      <c r="G1" s="26"/>
-      <c r="H1" s="26"/>
+      <c r="G1" s="34"/>
+      <c r="H1" s="34"/>
       <c r="I1" s="26"/>
       <c r="J1" s="27"/>
     </row>
     <row r="2" spans="1:10" ht="18" x14ac:dyDescent="0.25">
       <c r="A2" s="8"/>
-      <c r="B2" s="3"/>
-      <c r="C2" s="3">
+      <c r="B2" s="4"/>
+      <c r="C2" s="4">
         <v>8000</v>
       </c>
-      <c r="D2" s="3">
+      <c r="D2" s="4">
         <v>2</v>
       </c>
-      <c r="E2" s="3">
+      <c r="E2" s="4">
         <v>0.05</v>
       </c>
-      <c r="F2" s="3">
+      <c r="F2" s="4">
         <v>1.5E-3</v>
       </c>
-      <c r="G2" s="3"/>
-      <c r="H2" s="3"/>
+      <c r="G2" s="4"/>
+      <c r="H2" s="4"/>
       <c r="I2" s="3"/>
       <c r="J2" s="9"/>
     </row>
@@ -5198,47 +8251,47 @@
         <f>A1+1</f>
         <v>2</v>
       </c>
-      <c r="B3" s="18" t="s">
+      <c r="B3" s="23" t="s">
         <v>4</v>
       </c>
-      <c r="C3" s="18" t="s">
+      <c r="C3" s="23" t="s">
         <v>8</v>
       </c>
-      <c r="D3" s="18" t="s">
+      <c r="D3" s="23" t="s">
         <v>9</v>
       </c>
-      <c r="E3" s="18" t="s">
+      <c r="E3" s="23" t="s">
         <v>6</v>
       </c>
-      <c r="F3" s="18" t="s">
+      <c r="F3" s="23" t="s">
         <v>7</v>
       </c>
-      <c r="G3" s="18" t="s">
+      <c r="G3" s="23" t="s">
         <v>32</v>
       </c>
-      <c r="H3" s="18"/>
+      <c r="H3" s="23"/>
       <c r="I3" s="18"/>
       <c r="J3" s="29"/>
     </row>
     <row r="4" spans="1:10" ht="18" x14ac:dyDescent="0.25">
       <c r="A4" s="8"/>
-      <c r="B4" s="3"/>
-      <c r="C4" s="3">
+      <c r="B4" s="4"/>
+      <c r="C4" s="4">
         <v>8000</v>
       </c>
-      <c r="D4" s="3">
+      <c r="D4" s="4">
         <v>13000</v>
       </c>
-      <c r="E4" s="3">
+      <c r="E4" s="4">
         <v>4.7300000000000002E-2</v>
       </c>
-      <c r="F4" s="3">
+      <c r="F4" s="4">
         <v>0.1</v>
       </c>
-      <c r="G4" s="3">
+      <c r="G4" s="4">
         <v>0</v>
       </c>
-      <c r="H4" s="3"/>
+      <c r="H4" s="4"/>
       <c r="I4" s="3"/>
       <c r="J4" s="9"/>
     </row>
@@ -5247,47 +8300,47 @@
         <f>A3+1</f>
         <v>3</v>
       </c>
-      <c r="B5" s="18" t="s">
+      <c r="B5" s="23" t="s">
         <v>4</v>
       </c>
-      <c r="C5" s="18" t="s">
+      <c r="C5" s="23" t="s">
         <v>8</v>
       </c>
-      <c r="D5" s="18" t="s">
+      <c r="D5" s="23" t="s">
         <v>9</v>
       </c>
-      <c r="E5" s="18" t="s">
+      <c r="E5" s="23" t="s">
         <v>6</v>
       </c>
-      <c r="F5" s="18" t="s">
+      <c r="F5" s="23" t="s">
         <v>7</v>
       </c>
-      <c r="G5" s="18" t="s">
+      <c r="G5" s="23" t="s">
         <v>32</v>
       </c>
-      <c r="H5" s="18"/>
+      <c r="H5" s="23"/>
       <c r="I5" s="18"/>
       <c r="J5" s="29"/>
     </row>
     <row r="6" spans="1:10" ht="18" x14ac:dyDescent="0.25">
       <c r="A6" s="8"/>
-      <c r="B6" s="3"/>
-      <c r="C6" s="3">
+      <c r="B6" s="4"/>
+      <c r="C6" s="4">
         <v>13000</v>
       </c>
-      <c r="D6" s="3">
+      <c r="D6" s="4">
         <v>15000</v>
       </c>
-      <c r="E6" s="3">
+      <c r="E6" s="4">
         <v>0.1</v>
       </c>
-      <c r="F6" s="3">
+      <c r="F6" s="4">
         <v>0.2</v>
       </c>
-      <c r="G6" s="3">
+      <c r="G6" s="4">
         <v>0</v>
       </c>
-      <c r="H6" s="3"/>
+      <c r="H6" s="4"/>
       <c r="I6" s="3"/>
       <c r="J6" s="9"/>
     </row>
@@ -5295,43 +8348,43 @@
       <c r="A7" s="28">
         <v>6</v>
       </c>
-      <c r="B7" s="18" t="s">
+      <c r="B7" s="23" t="s">
         <v>10</v>
       </c>
-      <c r="C7" s="18" t="s">
+      <c r="C7" s="23" t="s">
         <v>5</v>
       </c>
-      <c r="D7" s="18" t="s">
+      <c r="D7" s="23" t="s">
         <v>17</v>
       </c>
-      <c r="E7" s="18" t="s">
+      <c r="E7" s="23" t="s">
         <v>11</v>
       </c>
-      <c r="F7" s="18" t="s">
+      <c r="F7" s="23" t="s">
         <v>33</v>
       </c>
-      <c r="G7" s="18"/>
-      <c r="H7" s="18"/>
+      <c r="G7" s="23"/>
+      <c r="H7" s="23"/>
       <c r="I7" s="18"/>
       <c r="J7" s="29"/>
     </row>
     <row r="8" spans="1:10" ht="18" x14ac:dyDescent="0.25">
       <c r="A8" s="8"/>
-      <c r="B8" s="3"/>
-      <c r="C8" s="3">
+      <c r="B8" s="4"/>
+      <c r="C8" s="4">
         <v>15000</v>
       </c>
-      <c r="D8" s="3">
+      <c r="D8" s="4">
         <v>100</v>
       </c>
-      <c r="E8" s="3">
+      <c r="E8" s="4">
         <v>0.2</v>
       </c>
-      <c r="F8" s="3">
+      <c r="F8" s="4">
         <v>0</v>
       </c>
-      <c r="G8" s="3"/>
-      <c r="H8" s="3"/>
+      <c r="G8" s="4"/>
+      <c r="H8" s="4"/>
       <c r="I8" s="3"/>
       <c r="J8" s="9"/>
     </row>
@@ -5339,40 +8392,40 @@
       <c r="A9" s="28">
         <v>7</v>
       </c>
-      <c r="B9" s="18" t="s">
+      <c r="B9" s="23" t="s">
         <v>12</v>
       </c>
-      <c r="C9" s="18" t="s">
+      <c r="C9" s="23" t="s">
         <v>5</v>
       </c>
-      <c r="D9" s="18" t="s">
+      <c r="D9" s="23" t="s">
         <v>13</v>
       </c>
-      <c r="E9" s="18" t="s">
+      <c r="E9" s="23" t="s">
         <v>34</v>
       </c>
-      <c r="F9" s="18"/>
-      <c r="G9" s="18"/>
-      <c r="H9" s="18"/>
+      <c r="F9" s="23"/>
+      <c r="G9" s="23"/>
+      <c r="H9" s="23"/>
       <c r="I9" s="18"/>
       <c r="J9" s="29"/>
     </row>
     <row r="10" spans="1:10" ht="18" x14ac:dyDescent="0.25">
       <c r="A10" s="8"/>
-      <c r="B10" s="3"/>
-      <c r="C10" s="14">
+      <c r="B10" s="4"/>
+      <c r="C10" s="35">
         <v>13000</v>
       </c>
-      <c r="D10" s="13">
+      <c r="D10" s="36">
         <f>10/60</f>
         <v>0.16666666666666666</v>
       </c>
       <c r="E10" s="3">
         <v>0</v>
       </c>
-      <c r="F10" s="3"/>
-      <c r="G10" s="3"/>
-      <c r="H10" s="3"/>
+      <c r="F10" s="4"/>
+      <c r="G10" s="4"/>
+      <c r="H10" s="4"/>
       <c r="I10" s="3"/>
       <c r="J10" s="9"/>
     </row>
@@ -7590,27 +10643,27 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="G15:G193 F15:F191 A15:E189 H1:J197">
-    <cfRule type="expression" dxfId="18" priority="11">
+    <cfRule type="expression" dxfId="37" priority="11">
       <formula>MOD(ROW(),2)=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A1 F1:G2 F9:G14 B1:E6 F3:F6 B7:G8">
-    <cfRule type="expression" dxfId="17" priority="6">
+    <cfRule type="expression" dxfId="36" priority="6">
       <formula>MOD(ROW(),2)=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B9:D10">
-    <cfRule type="expression" dxfId="16" priority="4">
+    <cfRule type="expression" dxfId="35" priority="4">
       <formula>MOD(ROW(),2)=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E9:E12">
-    <cfRule type="expression" dxfId="15" priority="3">
+    <cfRule type="expression" dxfId="34" priority="3">
       <formula>MOD(ROW(),2)=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G3:G6">
-    <cfRule type="expression" dxfId="14" priority="5">
+    <cfRule type="expression" dxfId="33" priority="5">
       <formula>MOD(ROW(),2)=0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -7618,7 +10671,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BC6C6E7F-A14C-C142-A4C3-77C3F7860513}">
   <dimension ref="A1:J200"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="18" x14ac:dyDescent="0.25"/>
@@ -10202,37 +13255,37 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A1:A2">
-    <cfRule type="expression" dxfId="13" priority="7">
+    <cfRule type="expression" dxfId="32" priority="7">
       <formula>MOD(ROW(),2)=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B1 D1:J1">
-    <cfRule type="expression" dxfId="12" priority="8">
+    <cfRule type="expression" dxfId="31" priority="8">
       <formula>MOD(ROW(),2)=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E14:E17">
-    <cfRule type="expression" dxfId="11" priority="1">
+    <cfRule type="expression" dxfId="30" priority="1">
       <formula>MOD(ROW(),2)=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F4:F5">
-    <cfRule type="expression" dxfId="10" priority="6">
+    <cfRule type="expression" dxfId="29" priority="6">
       <formula>MOD(ROW(),2)=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F10:F13">
-    <cfRule type="expression" dxfId="9" priority="2">
+    <cfRule type="expression" dxfId="28" priority="2">
       <formula>MOD(ROW(),2)=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G6:G9">
-    <cfRule type="expression" dxfId="8" priority="4">
+    <cfRule type="expression" dxfId="27" priority="4">
       <formula>MOD(ROW(),2)=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K1:XFD1 B2:XFD3 B4:E5 G4:XFD5 B6:F9 H6:XFD9 B10:E13 G10:XFD13 B14:D15 F14:XFD19 E20:XFD21 A22:XFD1048576">
-    <cfRule type="expression" dxfId="7" priority="10">
+    <cfRule type="expression" dxfId="26" priority="10">
       <formula>MOD(ROW(),2)=0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -10243,7 +13296,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{23008A42-2183-AF47-B42B-F6CD8E247DCD}">
   <dimension ref="A1:J200"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="18" x14ac:dyDescent="0.25"/>
@@ -12819,37 +15872,37 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A1:A2 F2:XFD3 B2:E11 H4:XFD7 G8:XFD11 F12:XFD19">
-    <cfRule type="expression" dxfId="6" priority="7">
+    <cfRule type="expression" dxfId="25" priority="7">
       <formula>MOD(ROW(),2)=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B1 D1:J1">
-    <cfRule type="expression" dxfId="5" priority="8">
+    <cfRule type="expression" dxfId="24" priority="8">
       <formula>MOD(ROW(),2)=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B12:D13">
-    <cfRule type="expression" dxfId="4" priority="2">
+    <cfRule type="expression" dxfId="23" priority="2">
       <formula>MOD(ROW(),2)=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E12:E15">
-    <cfRule type="expression" dxfId="3" priority="1">
+    <cfRule type="expression" dxfId="22" priority="1">
       <formula>MOD(ROW(),2)=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F4:F11">
-    <cfRule type="expression" dxfId="2" priority="3">
+    <cfRule type="expression" dxfId="21" priority="3">
       <formula>MOD(ROW(),2)=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G4:G7">
-    <cfRule type="expression" dxfId="1" priority="5">
+    <cfRule type="expression" dxfId="20" priority="5">
       <formula>MOD(ROW(),2)=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K1:XFD1 E20:XFD21 A22:XFD1048576">
-    <cfRule type="expression" dxfId="0" priority="9">
+    <cfRule type="expression" dxfId="19" priority="9">
       <formula>MOD(ROW(),2)=0</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>